<commit_message>
Add seven topics to the Databricks roadmap (91 topics, 12 phases)
Workspace objects and permissions; Photon and runtime selection; recovery,
replay and backfill; job concurrency and limits; autoscaling folded into
policies and pools; pipeline datasets widened to views and flows; and an
optional Azure networking phase of eight topics from notes section 20.
The plan gains guide chapter 23 (Azure networking). Import preview checked
again on a scratch database.
</commit_message>
<xml_diff>
--- a/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
+++ b/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\PrepBench\.claude\worktrees\databricks-research-1e243f\docs\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D771A2-9205-4096-9946-AFC171597DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34323425-181B-4317-BD98-F283F90A0AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="433">
   <si>
     <t>Phase</t>
   </si>
@@ -101,6 +101,18 @@
     <t>§17, §6.1</t>
   </si>
   <si>
+    <t>Workspace Objects and Permissions</t>
+  </si>
+  <si>
+    <t>Understand workspace-level assets (notebooks, folders, workspace files, jobs, pipelines, dashboards, queries) and that workspace access control lists, not Unity Catalog, govern them.</t>
+  </si>
+  <si>
+    <t>Sort ten objects into Unity Catalog securables and workspace assets, and say who controls access to each.</t>
+  </si>
+  <si>
+    <t>§6.1</t>
+  </si>
+  <si>
     <t>Product Names, Old and New</t>
   </si>
   <si>
@@ -488,9 +500,6 @@
     <t>Draw the hierarchy for one table, one volume and one external location, with who owns each.</t>
   </si>
   <si>
-    <t>§6.1</t>
-  </si>
-  <si>
     <t>Managed vs External Tables</t>
   </si>
   <si>
@@ -626,13 +635,22 @@
     <t>Say which access mode a shared team cluster and a single ML engineer's cluster should use.</t>
   </si>
   <si>
-    <t>Compute Policies and Pools</t>
-  </si>
-  <si>
-    <t>Understand admin compute policies that limit what users create, and pools that keep idle instances ready.</t>
-  </si>
-  <si>
-    <t>Design a policy that caps cluster size and forces auto termination for a data team.</t>
+    <t>Photon and Runtime Selection</t>
+  </si>
+  <si>
+    <t>Understand Databricks Runtime choice (latest for all-purpose, LTS for production jobs, versionless serverless) and Photon, the native vectorized engine on by default.</t>
+  </si>
+  <si>
+    <t>Choose a runtime for a production job and a development cluster, and say which workloads gain most from Photon.</t>
+  </si>
+  <si>
+    <t>Compute Policies, Pools and Autoscaling</t>
+  </si>
+  <si>
+    <t>Understand admin compute policies that limit what users create, autoscaling between minimum and maximum workers, and pools that keep idle instances ready (no DBUs while idle).</t>
+  </si>
+  <si>
+    <t>Design a policy that caps autoscaling and forces auto termination for a data team, and say when a pool is worth it.</t>
   </si>
   <si>
     <t>DBUs and Cost Levers</t>
@@ -794,16 +812,28 @@
     <t>§8, §2.7</t>
   </si>
   <si>
+    <t>Recovery, Replay and Backfill</t>
+  </si>
+  <si>
+    <t>Understand restart from a checkpoint vs starting fresh, full refresh and checkpoint reset in pipelines, RESTORE seen downstream as new data, and Auto Loader backfills.</t>
+  </si>
+  <si>
+    <t>Plan how to reprocess one bad week of data without duplicating rows downstream, naming each step's effect.</t>
+  </si>
+  <si>
+    <t>§8, §10, §2.2, §21.2</t>
+  </si>
+  <si>
     <t>10. Pipelines &amp; Orchestration</t>
   </si>
   <si>
-    <t>Streaming Tables vs Materialized Views</t>
-  </si>
-  <si>
-    <t>Master Lakeflow pipeline datasets: streaming tables (exactly-once, append-only sources) vs materialized views (recomputed to stay correct).</t>
-  </si>
-  <si>
-    <t>For five transformations, say which dataset type each should be and why.</t>
+    <t>Pipeline Datasets and Flows</t>
+  </si>
+  <si>
+    <t>Master Lakeflow pipeline datasets (streaming tables, materialized views, views) and flows (append, update, AUTO CDC, materialized view) and how dependencies form the pipeline graph.</t>
+  </si>
+  <si>
+    <t>For five transformations, say which dataset type each should be and why, and which flow writes it.</t>
   </si>
   <si>
     <t>§10</t>
@@ -857,6 +887,15 @@
     <t>Configure a cleanup task that runs even when an upstream task fails, and a retry on a flaky task.</t>
   </si>
   <si>
+    <t>Job Concurrency and Limits</t>
+  </si>
+  <si>
+    <t>Understand one run at a time by default, maximum concurrent runs (runs beyond it are skipped), and workspace limits such as 2,000 concurrent task runs.</t>
+  </si>
+  <si>
+    <t>Explain what happens when an hourly job's run takes 90 minutes, and how to change it.</t>
+  </si>
+  <si>
     <t>Triggers and Repair Runs</t>
   </si>
   <si>
@@ -875,7 +914,97 @@
     <t>Design how an ADF pipeline triggers a Databricks job and reads back its result.</t>
   </si>
   <si>
-    <t>11. Operate, Deploy &amp; Capstone</t>
+    <t>11. Azure Networking for Databricks</t>
+  </si>
+  <si>
+    <t>Three Network Connections</t>
+  </si>
+  <si>
+    <t>Understand the three connections secured separately: users to Databricks, control plane to classic compute, and serverless compute to your resources.</t>
+  </si>
+  <si>
+    <t>Draw the three connections for one workspace and name a control for each.</t>
+  </si>
+  <si>
+    <t>§20.1</t>
+  </si>
+  <si>
+    <t>Serverless vs Hybrid Workspaces</t>
+  </si>
+  <si>
+    <t>Understand serverless workspaces (default storage, serverless compute) vs hybrid (classic) workspaces in your subscription, and who may create one.</t>
+  </si>
+  <si>
+    <t>Choose a workspace type for two teams with different needs and justify it.</t>
+  </si>
+  <si>
+    <t>§20.2</t>
+  </si>
+  <si>
+    <t>VNet Injection and Subnet Sizing</t>
+  </si>
+  <si>
+    <t>Master VNet injection: same region and subscription, /16 to /24 VNet, two dedicated subnets (container and host, /26 recommended), two IPs per node, ranges fixed after deployment.</t>
+  </si>
+  <si>
+    <t>Size a VNet and its two subnets for a 100-node peak and show the arithmetic.</t>
+  </si>
+  <si>
+    <t>§20.3</t>
+  </si>
+  <si>
+    <t>Subnet Delegation and NSG Rules</t>
+  </si>
+  <si>
+    <t>Understand subnet delegation to Databricks, the managed NSG rules and their ports, and why they must not be modified.</t>
+  </si>
+  <si>
+    <t>Explain which outbound ports a VNet-injected workspace needs and what each one is for.</t>
+  </si>
+  <si>
+    <t>Secure Cluster Connectivity and Egress</t>
+  </si>
+  <si>
+    <t>Master secure cluster connectivity (no public IPs, outbound relay on 443), NAT gateway egress, and the March 2026 change to default outbound access.</t>
+  </si>
+  <si>
+    <t>Explain why a new workspace's clusters can't reach the internet without a NAT gateway, and how to fix it.</t>
+  </si>
+  <si>
+    <t>§20.4</t>
+  </si>
+  <si>
+    <t>Private Link: Three Kinds</t>
+  </si>
+  <si>
+    <t>Understand inbound (front-end), outbound (serverless) and classic (back-end) Private Link, their prerequisites and endpoints, and complete private isolation.</t>
+  </si>
+  <si>
+    <t>Pick the Private Link setup for a bank that forbids any public path, and list the endpoints it needs.</t>
+  </si>
+  <si>
+    <t>§20.5</t>
+  </si>
+  <si>
+    <t>Browser Authentication and the Transit VNet</t>
+  </si>
+  <si>
+    <t>Understand the browser_authentication endpoint (one per region and DNS zone), the private web auth workspace, and transit vs workspace VNets.</t>
+  </si>
+  <si>
+    <t>Explain why deleting one workspace could break SSO for every private workspace in the region.</t>
+  </si>
+  <si>
+    <t>Serverless Connectivity and Storage Firewalls</t>
+  </si>
+  <si>
+    <t>Understand NCCs and serverless private endpoints, service endpoints, and storage firewalls with network security perimeters and the AzureDatabricksServerless tag.</t>
+  </si>
+  <si>
+    <t>Diagnose a serverless job getting 403 Forbidden from a firewalled ADLS account and give the fix.</t>
+  </si>
+  <si>
+    <t>12. Operate, Deploy &amp; Capstone</t>
   </si>
   <si>
     <t>System Tables and Monitoring</t>
@@ -944,7 +1073,7 @@
     <t>Run the pipeline in Free Edition, grant a reader group on gold, and explain every design choice to a reviewer.</t>
   </si>
   <si>
-    <t>1-22</t>
+    <t>1-23</t>
   </si>
   <si>
     <t>all</t>
@@ -1586,7 +1715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1701,7 +1830,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="56" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -1727,7 +1856,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="56" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1744,7 +1873,7 @@
         <v>27</v>
       </c>
       <c r="F6" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
@@ -1753,35 +1882,35 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="F7" s="3">
         <v>2</v>
       </c>
       <c r="G7" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="42" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="B8" s="2">
         <v>7</v>
@@ -1796,7 +1925,7 @@
         <v>36</v>
       </c>
       <c r="F8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" s="2">
         <v>2</v>
@@ -1805,9 +1934,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B9" s="3">
         <v>8</v>
@@ -1831,9 +1960,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2">
         <v>9</v>
@@ -1859,7 +1988,7 @@
     </row>
     <row r="11" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
@@ -1874,7 +2003,7 @@
         <v>48</v>
       </c>
       <c r="F11" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="3">
         <v>2</v>
@@ -1885,7 +2014,7 @@
     </row>
     <row r="12" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2">
         <v>11</v>
@@ -1906,12 +2035,12 @@
         <v>2</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B13" s="3">
         <v>12</v>
@@ -1929,15 +2058,15 @@
         <v>2</v>
       </c>
       <c r="G13" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H13" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="42" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="B14" s="2">
         <v>13</v>
@@ -1952,30 +2081,30 @@
         <v>60</v>
       </c>
       <c r="F14" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" s="2">
         <v>3</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F15" s="3">
         <v>3</v>
@@ -1984,12 +2113,12 @@
         <v>3</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -2013,9 +2142,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B17" s="3">
         <v>16</v>
@@ -2041,7 +2170,7 @@
     </row>
     <row r="18" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2">
         <v>17</v>
@@ -2056,70 +2185,70 @@
         <v>75</v>
       </c>
       <c r="F18" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" s="2">
         <v>3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B19" s="3">
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F19" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" s="3">
         <v>3</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2">
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F20" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="2">
         <v>3</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B21" s="3">
         <v>20</v>
@@ -2145,33 +2274,33 @@
     </row>
     <row r="22" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="B22" s="2">
         <v>21</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2">
+        <v>3</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="F22" s="2">
-        <v>1</v>
-      </c>
-      <c r="G22" s="2">
-        <v>4</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B23" s="3">
         <v>22</v>
@@ -2186,30 +2315,30 @@
         <v>94</v>
       </c>
       <c r="F23" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="3">
         <v>4</v>
       </c>
       <c r="H23" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="42" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="B24" s="2">
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F24" s="2">
         <v>2</v>
@@ -2218,24 +2347,24 @@
         <v>4</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B25" s="3">
         <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F25" s="3">
         <v>2</v>
@@ -2244,12 +2373,12 @@
         <v>4</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B26" s="2">
         <v>25</v>
@@ -2270,38 +2399,38 @@
         <v>4</v>
       </c>
       <c r="H26" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="28" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
-        <v>87</v>
       </c>
       <c r="B27" s="3">
         <v>26</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F27" s="3">
         <v>2</v>
       </c>
       <c r="G27" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B28" s="2">
         <v>27</v>
@@ -2322,38 +2451,38 @@
         <v>5</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B29" s="3">
         <v>28</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F29" s="3">
+        <v>2</v>
+      </c>
+      <c r="G29" s="3">
+        <v>5</v>
+      </c>
+      <c r="H29" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F29" s="3">
-        <v>4</v>
-      </c>
-      <c r="G29" s="3">
-        <v>6</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B30" s="2">
         <v>29</v>
@@ -2368,7 +2497,7 @@
         <v>118</v>
       </c>
       <c r="F30" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G30" s="2">
         <v>6</v>
@@ -2379,33 +2508,33 @@
     </row>
     <row r="31" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="B31" s="3">
         <v>30</v>
       </c>
       <c r="C31" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="F31" s="3">
+        <v>3</v>
+      </c>
+      <c r="G31" s="3">
+        <v>6</v>
+      </c>
+      <c r="H31" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="F31" s="3">
-        <v>2</v>
-      </c>
-      <c r="G31" s="3">
-        <v>7</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B32" s="2">
         <v>31</v>
@@ -2431,7 +2560,7 @@
     </row>
     <row r="33" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B33" s="3">
         <v>32</v>
@@ -2452,90 +2581,90 @@
         <v>7</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B34" s="2">
         <v>33</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F34" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G34" s="2">
         <v>7</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B35" s="3">
         <v>34</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" s="3">
         <v>7</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B36" s="2">
         <v>35</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F36" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="2">
         <v>7</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B37" s="3">
         <v>36</v>
@@ -2550,7 +2679,7 @@
         <v>144</v>
       </c>
       <c r="F37" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" s="3">
         <v>7</v>
@@ -2561,33 +2690,33 @@
     </row>
     <row r="38" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="B38" s="2">
         <v>37</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="F38" s="2">
         <v>2</v>
       </c>
       <c r="G38" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H38" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="28" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>146</v>
       </c>
       <c r="B39" s="3">
         <v>38</v>
@@ -2602,174 +2731,174 @@
         <v>153</v>
       </c>
       <c r="F39" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>154</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B40" s="2">
         <v>39</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="E40" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="F40" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G40" s="2">
         <v>9</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B41" s="3">
         <v>40</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>161</v>
-      </c>
       <c r="F41" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G41" s="3">
         <v>9</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B42" s="2">
         <v>41</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="F42" s="2">
         <v>3</v>
       </c>
       <c r="G42" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B43" s="3">
         <v>42</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D43" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="E43" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>169</v>
-      </c>
       <c r="F43" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G43" s="3">
         <v>10</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B44" s="2">
         <v>43</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E44" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="F44" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G44" s="2">
         <v>10</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B45" s="3">
         <v>44</v>
       </c>
       <c r="C45" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="E45" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E45" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="F45" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G45" s="3">
         <v>10</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B46" s="2">
         <v>45</v>
@@ -2790,64 +2919,64 @@
         <v>10</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="B47" s="3">
         <v>46</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>185</v>
       </c>
       <c r="F47" s="3">
         <v>2</v>
       </c>
       <c r="G47" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B48" s="2">
         <v>47</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>189</v>
-      </c>
       <c r="F48" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="2">
         <v>11</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B49" s="3">
         <v>48</v>
@@ -2868,12 +2997,12 @@
         <v>11</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B50" s="2">
         <v>49</v>
@@ -2894,12 +3023,12 @@
         <v>11</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B51" s="3">
         <v>50</v>
@@ -2914,18 +3043,18 @@
         <v>198</v>
       </c>
       <c r="F51" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51" s="3">
         <v>11</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B52" s="2">
         <v>51</v>
@@ -2946,76 +3075,76 @@
         <v>11</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="B53" s="3">
         <v>52</v>
       </c>
       <c r="C53" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="E53" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="E53" s="3" t="s">
-        <v>205</v>
-      </c>
       <c r="F53" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G53" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="B54" s="2">
         <v>53</v>
       </c>
       <c r="C54" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="F54" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G54" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B55" s="3">
         <v>54</v>
       </c>
       <c r="C55" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="E55" s="3" t="s">
         <v>211</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>212</v>
       </c>
       <c r="F55" s="3">
         <v>3</v>
@@ -3024,12 +3153,12 @@
         <v>12</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B56" s="2">
         <v>55</v>
@@ -3047,15 +3176,15 @@
         <v>3</v>
       </c>
       <c r="G56" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B57" s="3">
         <v>56</v>
@@ -3073,15 +3202,15 @@
         <v>3</v>
       </c>
       <c r="G57" s="3">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B58" s="2">
         <v>57</v>
@@ -3099,15 +3228,15 @@
         <v>3</v>
       </c>
       <c r="G58" s="2">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B59" s="3">
         <v>58</v>
@@ -3122,186 +3251,186 @@
         <v>224</v>
       </c>
       <c r="F59" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G59" s="3">
         <v>19</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="B60" s="2">
         <v>59</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D60" s="2" t="s">
+      <c r="E60" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="E60" s="2" t="s">
-        <v>228</v>
-      </c>
       <c r="F60" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G60" s="2">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="B61" s="3">
         <v>60</v>
       </c>
       <c r="C61" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E61" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>232</v>
       </c>
       <c r="F61" s="3">
         <v>2</v>
       </c>
       <c r="G61" s="3">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B62" s="2">
         <v>61</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="F62" s="2">
+        <v>2</v>
+      </c>
+      <c r="G62" s="2">
+        <v>14</v>
+      </c>
+      <c r="H62" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F62" s="2">
-        <v>3</v>
-      </c>
-      <c r="G62" s="2">
-        <v>15</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B63" s="3">
         <v>62</v>
       </c>
       <c r="C63" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E63" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D63" s="3" t="s">
+      <c r="F63" s="3">
+        <v>2</v>
+      </c>
+      <c r="G63" s="3">
+        <v>14</v>
+      </c>
+      <c r="H63" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="E63" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="F63" s="3">
-        <v>3</v>
-      </c>
-      <c r="G63" s="3">
-        <v>15</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B64" s="2">
         <v>63</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="E64" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>243</v>
       </c>
       <c r="F64" s="2">
         <v>3</v>
       </c>
       <c r="G64" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B65" s="3">
         <v>64</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D65" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="E65" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>247</v>
       </c>
       <c r="F65" s="3">
         <v>3</v>
       </c>
       <c r="G65" s="3">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B66" s="2">
         <v>65</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="F66" s="2">
         <v>3</v>
@@ -3310,90 +3439,90 @@
         <v>16</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>252</v>
+        <v>231</v>
       </c>
       <c r="B67" s="3">
         <v>66</v>
       </c>
       <c r="C67" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E67" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="F67" s="3">
         <v>3</v>
       </c>
       <c r="G67" s="3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
-        <v>252</v>
+        <v>231</v>
       </c>
       <c r="B68" s="2">
         <v>67</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F68" s="2">
+        <v>3</v>
+      </c>
+      <c r="G68" s="2">
+        <v>16</v>
+      </c>
+      <c r="H68" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="F68" s="2">
-        <v>2</v>
-      </c>
-      <c r="G68" s="2">
-        <v>17</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    </row>
+    <row r="69" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>252</v>
+        <v>231</v>
       </c>
       <c r="B69" s="3">
         <v>68</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E69" s="3" t="s">
         <v>260</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>262</v>
       </c>
       <c r="F69" s="3">
         <v>3</v>
       </c>
       <c r="G69" s="3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B70" s="2">
         <v>69</v>
@@ -3408,44 +3537,44 @@
         <v>265</v>
       </c>
       <c r="F70" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G70" s="2">
         <v>17</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B71" s="3">
         <v>70</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="F71" s="3">
+        <v>2</v>
+      </c>
+      <c r="G71" s="3">
+        <v>17</v>
+      </c>
+      <c r="H71" s="3" t="s">
         <v>266</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="F71" s="3">
-        <v>3</v>
-      </c>
-      <c r="G71" s="3">
-        <v>18</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B72" s="2">
         <v>71</v>
@@ -3460,18 +3589,18 @@
         <v>272</v>
       </c>
       <c r="F72" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B73" s="3">
         <v>72</v>
@@ -3489,15 +3618,15 @@
         <v>2</v>
       </c>
       <c r="G73" s="3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B74" s="2">
         <v>73</v>
@@ -3512,18 +3641,18 @@
         <v>278</v>
       </c>
       <c r="F74" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G74" s="2">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>16</v>
+        <v>279</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="B75" s="3">
         <v>74</v>
@@ -3538,152 +3667,464 @@
         <v>282</v>
       </c>
       <c r="F75" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G75" s="3">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="B76" s="2">
         <v>75</v>
       </c>
       <c r="C76" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="E76" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="E76" s="2" t="s">
-        <v>286</v>
-      </c>
       <c r="F76" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G76" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="B77" s="3">
         <v>76</v>
       </c>
       <c r="C77" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E77" s="3" t="s">
         <v>288</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="E77" s="3" t="s">
-        <v>290</v>
       </c>
       <c r="F77" s="3">
         <v>2</v>
       </c>
       <c r="G77" s="3">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="B78" s="2">
         <v>77</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="F78" s="2">
+        <v>2</v>
+      </c>
+      <c r="G78" s="2">
+        <v>22</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A79" s="3" t="s">
         <v>292</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F78" s="2">
-        <v>1</v>
-      </c>
-      <c r="G78" s="2">
-        <v>21</v>
-      </c>
-      <c r="H78" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" ht="28" x14ac:dyDescent="0.35">
-      <c r="A79" s="3" t="s">
-        <v>279</v>
       </c>
       <c r="B79" s="3">
         <v>78</v>
       </c>
       <c r="C79" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="F79" s="3">
+        <v>2</v>
+      </c>
+      <c r="G79" s="3">
+        <v>23</v>
+      </c>
+      <c r="H79" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="D79" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E79" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="F79" s="3">
-        <v>4</v>
-      </c>
-      <c r="G79" s="3">
-        <v>21</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    </row>
+    <row r="80" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="B80" s="2">
         <v>79</v>
       </c>
       <c r="C80" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="F80" s="2">
+        <v>1</v>
+      </c>
+      <c r="G80" s="2">
+        <v>23</v>
+      </c>
+      <c r="H80" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E80" s="2" t="s">
+    </row>
+    <row r="81" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A81" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B81" s="3">
+        <v>80</v>
+      </c>
+      <c r="C81" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="F80" s="2">
+      <c r="D81" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="F81" s="3">
+        <v>3</v>
+      </c>
+      <c r="G81" s="3">
+        <v>23</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A82" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B82" s="2">
+        <v>81</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F82" s="2">
+        <v>2</v>
+      </c>
+      <c r="G82" s="2">
+        <v>23</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B83" s="3">
+        <v>82</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="F83" s="3">
+        <v>2</v>
+      </c>
+      <c r="G83" s="3">
+        <v>23</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B84" s="2">
+        <v>83</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F84" s="2">
+        <v>3</v>
+      </c>
+      <c r="G84" s="2">
+        <v>23</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A85" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B85" s="3">
+        <v>84</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="F85" s="3">
+        <v>2</v>
+      </c>
+      <c r="G85" s="3">
+        <v>23</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B86" s="2">
+        <v>85</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F86" s="2">
+        <v>2</v>
+      </c>
+      <c r="G86" s="2">
+        <v>23</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A87" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B87" s="3">
+        <v>86</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="F87" s="3">
+        <v>3</v>
+      </c>
+      <c r="G87" s="3">
+        <v>20</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B88" s="2">
+        <v>87</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F88" s="2">
+        <v>2</v>
+      </c>
+      <c r="G88" s="2">
+        <v>20</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A89" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B89" s="3">
+        <v>88</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="F89" s="3">
+        <v>2</v>
+      </c>
+      <c r="G89" s="3">
+        <v>21</v>
+      </c>
+      <c r="H89" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A90" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B90" s="2">
+        <v>89</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F90" s="2">
+        <v>1</v>
+      </c>
+      <c r="G90" s="2">
+        <v>21</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A91" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B91" s="3">
+        <v>90</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="F91" s="3">
+        <v>4</v>
+      </c>
+      <c r="G91" s="3">
+        <v>21</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A92" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B92" s="2">
+        <v>91</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F92" s="2">
         <v>10</v>
       </c>
-      <c r="G80" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H80" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="81" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C81" s="4" t="s">
-        <v>304</v>
-      </c>
-      <c r="F81" s="4">
-        <f>SUM(F2:F80)</f>
-        <v>193</v>
+      <c r="G92" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C93" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="F93" s="4">
+        <f>SUM(F2:F92)</f>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3693,7 +4134,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3707,45 +4148,45 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>305</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>306</v>
+        <v>349</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>307</v>
+        <v>350</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>308</v>
+        <v>351</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>310</v>
+        <v>353</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <f>COUNTA(B6:B84)</f>
-        <v>79</v>
+        <f>COUNTA(B6:B96)</f>
+        <v>91</v>
       </c>
       <c r="B3" s="5">
-        <f>COUNTIF(D6:D84,"Completed")</f>
+        <f>COUNTIF(D6:D96,"Completed")</f>
         <v>0</v>
       </c>
       <c r="C3" s="5">
-        <f>COUNTIF(D6:D84,"In Progress")</f>
+        <f>COUNTIF(D6:D96,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="D3" s="5">
-        <f>COUNTIF(D6:D84,"Not Started")</f>
-        <v>79</v>
+        <f>COUNTIF(D6:D96,"Not Started")</f>
+        <v>91</v>
       </c>
       <c r="E3" s="6">
-        <f>AVERAGE(E6:E84)/100</f>
+        <f>AVERAGE(E6:E96)/100</f>
         <v>0</v>
       </c>
     </row>
@@ -3760,19 +4201,19 @@
         <v>0</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>311</v>
+        <v>354</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>312</v>
+        <v>355</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>313</v>
+        <v>356</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>314</v>
+        <v>357</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>315</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -3788,7 +4229,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E6" s="2">
         <v>0</v>
@@ -3810,7 +4251,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E7" s="3">
         <v>0</v>
@@ -3832,7 +4273,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E8" s="2">
         <v>0</v>
@@ -3847,14 +4288,14 @@
       </c>
       <c r="B9" s="3" t="str">
         <f>'Databricks Master Syllabus'!C5</f>
-        <v>Product Names, Old and New</v>
+        <v>Workspace Objects and Permissions</v>
       </c>
       <c r="C9" s="3" t="str">
         <f>'Databricks Master Syllabus'!A5</f>
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E9" s="3">
         <v>0</v>
@@ -3869,14 +4310,14 @@
       </c>
       <c r="B10" s="2" t="str">
         <f>'Databricks Master Syllabus'!C6</f>
-        <v>Databricks Free Edition Setup</v>
+        <v>Product Names, Old and New</v>
       </c>
       <c r="C10" s="2" t="str">
         <f>'Databricks Master Syllabus'!A6</f>
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E10" s="2">
         <v>0</v>
@@ -3891,14 +4332,14 @@
       </c>
       <c r="B11" s="3" t="str">
         <f>'Databricks Master Syllabus'!C7</f>
-        <v>Columnar Storage</v>
+        <v>Databricks Free Edition Setup</v>
       </c>
       <c r="C11" s="3" t="str">
         <f>'Databricks Master Syllabus'!A7</f>
-        <v>2. Parquet: The File Format</v>
+        <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E11" s="3">
         <v>0</v>
@@ -3913,14 +4354,14 @@
       </c>
       <c r="B12" s="2" t="str">
         <f>'Databricks Master Syllabus'!C8</f>
-        <v>Parquet File Anatomy</v>
+        <v>Columnar Storage</v>
       </c>
       <c r="C12" s="2" t="str">
         <f>'Databricks Master Syllabus'!A8</f>
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
@@ -3935,14 +4376,14 @@
       </c>
       <c r="B13" s="3" t="str">
         <f>'Databricks Master Syllabus'!C9</f>
-        <v>Statistics, Page Index and Bloom Filters</v>
+        <v>Parquet File Anatomy</v>
       </c>
       <c r="C13" s="3" t="str">
         <f>'Databricks Master Syllabus'!A9</f>
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E13" s="3">
         <v>0</v>
@@ -3957,14 +4398,14 @@
       </c>
       <c r="B14" s="2" t="str">
         <f>'Databricks Master Syllabus'!C10</f>
-        <v>Types, Encodings and Compression</v>
+        <v>Statistics, Page Index and Bloom Filters</v>
       </c>
       <c r="C14" s="2" t="str">
         <f>'Databricks Master Syllabus'!A10</f>
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E14" s="2">
         <v>0</v>
@@ -3979,14 +4420,14 @@
       </c>
       <c r="B15" s="3" t="str">
         <f>'Databricks Master Syllabus'!C11</f>
-        <v>Parquet in Spark</v>
+        <v>Types, Encodings and Compression</v>
       </c>
       <c r="C15" s="3" t="str">
         <f>'Databricks Master Syllabus'!A11</f>
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E15" s="3">
         <v>0</v>
@@ -4001,14 +4442,14 @@
       </c>
       <c r="B16" s="2" t="str">
         <f>'Databricks Master Syllabus'!C12</f>
-        <v>Hive-Style Partitioning and Small Files</v>
+        <v>Parquet in Spark</v>
       </c>
       <c r="C16" s="2" t="str">
         <f>'Databricks Master Syllabus'!A12</f>
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E16" s="2">
         <v>0</v>
@@ -4023,14 +4464,14 @@
       </c>
       <c r="B17" s="3" t="str">
         <f>'Databricks Master Syllabus'!C13</f>
-        <v>Delta Lake = Parquet + Transaction Log</v>
+        <v>Hive-Style Partitioning and Small Files</v>
       </c>
       <c r="C17" s="3" t="str">
         <f>'Databricks Master Syllabus'!A13</f>
-        <v>3. Delta Lake Internals</v>
+        <v>2. Parquet: The File Format</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -4045,14 +4486,14 @@
       </c>
       <c r="B18" s="2" t="str">
         <f>'Databricks Master Syllabus'!C14</f>
-        <v>Commit Files in _delta_log</v>
+        <v>Delta Lake = Parquet + Transaction Log</v>
       </c>
       <c r="C18" s="2" t="str">
         <f>'Databricks Master Syllabus'!A14</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E18" s="2">
         <v>0</v>
@@ -4067,14 +4508,14 @@
       </c>
       <c r="B19" s="3" t="str">
         <f>'Databricks Master Syllabus'!C15</f>
-        <v>Log Actions</v>
+        <v>Commit Files in _delta_log</v>
       </c>
       <c r="C19" s="3" t="str">
         <f>'Databricks Master Syllabus'!A15</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E19" s="3">
         <v>0</v>
@@ -4089,14 +4530,14 @@
       </c>
       <c r="B20" s="2" t="str">
         <f>'Databricks Master Syllabus'!C16</f>
-        <v>Snapshots, Tombstones and Log Replay</v>
+        <v>Log Actions</v>
       </c>
       <c r="C20" s="2" t="str">
         <f>'Databricks Master Syllabus'!A16</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E20" s="2">
         <v>0</v>
@@ -4111,14 +4552,14 @@
       </c>
       <c r="B21" s="3" t="str">
         <f>'Databricks Master Syllabus'!C17</f>
-        <v>Checkpoints and _last_checkpoint</v>
+        <v>Snapshots, Tombstones and Log Replay</v>
       </c>
       <c r="C21" s="3" t="str">
         <f>'Databricks Master Syllabus'!A17</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E21" s="3">
         <v>0</v>
@@ -4133,14 +4574,14 @@
       </c>
       <c r="B22" s="2" t="str">
         <f>'Databricks Master Syllabus'!C18</f>
-        <v>Optimistic Concurrency and Write Conflicts</v>
+        <v>Checkpoints and _last_checkpoint</v>
       </c>
       <c r="C22" s="2" t="str">
         <f>'Databricks Master Syllabus'!A18</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E22" s="2">
         <v>0</v>
@@ -4155,14 +4596,14 @@
       </c>
       <c r="B23" s="3" t="str">
         <f>'Databricks Master Syllabus'!C19</f>
-        <v>Isolation Levels and Transaction Scope</v>
+        <v>Optimistic Concurrency and Write Conflicts</v>
       </c>
       <c r="C23" s="3" t="str">
         <f>'Databricks Master Syllabus'!A19</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E23" s="3">
         <v>0</v>
@@ -4177,14 +4618,14 @@
       </c>
       <c r="B24" s="2" t="str">
         <f>'Databricks Master Syllabus'!C20</f>
-        <v>Protocol Versions and Table Features</v>
+        <v>Isolation Levels and Transaction Scope</v>
       </c>
       <c r="C24" s="2" t="str">
         <f>'Databricks Master Syllabus'!A20</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E24" s="2">
         <v>0</v>
@@ -4199,14 +4640,14 @@
       </c>
       <c r="B25" s="3" t="str">
         <f>'Databricks Master Syllabus'!C21</f>
-        <v>Idempotent Writes with Transaction Identifiers</v>
+        <v>Protocol Versions and Table Features</v>
       </c>
       <c r="C25" s="3" t="str">
         <f>'Databricks Master Syllabus'!A21</f>
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E25" s="3">
         <v>0</v>
@@ -4221,14 +4662,14 @@
       </c>
       <c r="B26" s="2" t="str">
         <f>'Databricks Master Syllabus'!C22</f>
-        <v>Table History</v>
+        <v>Idempotent Writes with Transaction Identifiers</v>
       </c>
       <c r="C26" s="2" t="str">
         <f>'Databricks Master Syllabus'!A22</f>
-        <v>4. Delta Lake Operations</v>
+        <v>3. Delta Lake Internals</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
@@ -4243,14 +4684,14 @@
       </c>
       <c r="B27" s="3" t="str">
         <f>'Databricks Master Syllabus'!C23</f>
-        <v>Time Travel</v>
+        <v>Table History</v>
       </c>
       <c r="C27" s="3" t="str">
         <f>'Databricks Master Syllabus'!A23</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E27" s="3">
         <v>0</v>
@@ -4265,14 +4706,14 @@
       </c>
       <c r="B28" s="2" t="str">
         <f>'Databricks Master Syllabus'!C24</f>
-        <v>Log Retention vs Deleted-File Retention</v>
+        <v>Time Travel</v>
       </c>
       <c r="C28" s="2" t="str">
         <f>'Databricks Master Syllabus'!A24</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E28" s="2">
         <v>0</v>
@@ -4287,14 +4728,14 @@
       </c>
       <c r="B29" s="3" t="str">
         <f>'Databricks Master Syllabus'!C25</f>
-        <v>VACUUM</v>
+        <v>Log Retention vs Deleted-File Retention</v>
       </c>
       <c r="C29" s="3" t="str">
         <f>'Databricks Master Syllabus'!A25</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E29" s="3">
         <v>0</v>
@@ -4309,14 +4750,14 @@
       </c>
       <c r="B30" s="2" t="str">
         <f>'Databricks Master Syllabus'!C26</f>
-        <v>RESTORE</v>
+        <v>VACUUM</v>
       </c>
       <c r="C30" s="2" t="str">
         <f>'Databricks Master Syllabus'!A26</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E30" s="2">
         <v>0</v>
@@ -4331,14 +4772,14 @@
       </c>
       <c r="B31" s="3" t="str">
         <f>'Databricks Master Syllabus'!C27</f>
-        <v>Schema Enforcement</v>
+        <v>RESTORE</v>
       </c>
       <c r="C31" s="3" t="str">
         <f>'Databricks Master Syllabus'!A27</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E31" s="3">
         <v>0</v>
@@ -4353,14 +4794,14 @@
       </c>
       <c r="B32" s="2" t="str">
         <f>'Databricks Master Syllabus'!C28</f>
-        <v>Schema Evolution</v>
+        <v>Schema Enforcement</v>
       </c>
       <c r="C32" s="2" t="str">
         <f>'Databricks Master Syllabus'!A28</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -4375,14 +4816,14 @@
       </c>
       <c r="B33" s="3" t="str">
         <f>'Databricks Master Syllabus'!C29</f>
-        <v>MERGE Upserts</v>
+        <v>Schema Evolution</v>
       </c>
       <c r="C33" s="3" t="str">
         <f>'Databricks Master Syllabus'!A29</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E33" s="3">
         <v>0</v>
@@ -4397,14 +4838,14 @@
       </c>
       <c r="B34" s="2" t="str">
         <f>'Databricks Master Syllabus'!C30</f>
-        <v>Change Data Feed</v>
+        <v>MERGE Upserts</v>
       </c>
       <c r="C34" s="2" t="str">
         <f>'Databricks Master Syllabus'!A30</f>
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E34" s="2">
         <v>0</v>
@@ -4419,14 +4860,14 @@
       </c>
       <c r="B35" s="3" t="str">
         <f>'Databricks Master Syllabus'!C31</f>
-        <v>OPTIMIZE and Compaction</v>
+        <v>Change Data Feed</v>
       </c>
       <c r="C35" s="3" t="str">
         <f>'Databricks Master Syllabus'!A31</f>
-        <v>5. Data Layout &amp; Table Optimization</v>
+        <v>4. Delta Lake Operations</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E35" s="3">
         <v>0</v>
@@ -4441,14 +4882,14 @@
       </c>
       <c r="B36" s="2" t="str">
         <f>'Databricks Master Syllabus'!C32</f>
-        <v>Data Skipping and File Statistics</v>
+        <v>OPTIMIZE and Compaction</v>
       </c>
       <c r="C36" s="2" t="str">
         <f>'Databricks Master Syllabus'!A32</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E36" s="2">
         <v>0</v>
@@ -4463,14 +4904,14 @@
       </c>
       <c r="B37" s="3" t="str">
         <f>'Databricks Master Syllabus'!C33</f>
-        <v>Z-Order</v>
+        <v>Data Skipping and File Statistics</v>
       </c>
       <c r="C37" s="3" t="str">
         <f>'Databricks Master Syllabus'!A33</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E37" s="3">
         <v>0</v>
@@ -4485,14 +4926,14 @@
       </c>
       <c r="B38" s="2" t="str">
         <f>'Databricks Master Syllabus'!C34</f>
-        <v>Liquid Clustering</v>
+        <v>Z-Order</v>
       </c>
       <c r="C38" s="2" t="str">
         <f>'Databricks Master Syllabus'!A34</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E38" s="2">
         <v>0</v>
@@ -4507,14 +4948,14 @@
       </c>
       <c r="B39" s="3" t="str">
         <f>'Databricks Master Syllabus'!C35</f>
-        <v>Deletion Vectors</v>
+        <v>Liquid Clustering</v>
       </c>
       <c r="C39" s="3" t="str">
         <f>'Databricks Master Syllabus'!A35</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E39" s="3">
         <v>0</v>
@@ -4529,14 +4970,14 @@
       </c>
       <c r="B40" s="2" t="str">
         <f>'Databricks Master Syllabus'!C36</f>
-        <v>Predictive Optimization</v>
+        <v>Deletion Vectors</v>
       </c>
       <c r="C40" s="2" t="str">
         <f>'Databricks Master Syllabus'!A36</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E40" s="2">
         <v>0</v>
@@ -4551,14 +4992,14 @@
       </c>
       <c r="B41" s="3" t="str">
         <f>'Databricks Master Syllabus'!C37</f>
-        <v>Partitioning on Databricks</v>
+        <v>Predictive Optimization</v>
       </c>
       <c r="C41" s="3" t="str">
         <f>'Databricks Master Syllabus'!A37</f>
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E41" s="3">
         <v>0</v>
@@ -4573,14 +5014,14 @@
       </c>
       <c r="B42" s="2" t="str">
         <f>'Databricks Master Syllabus'!C38</f>
-        <v>Unity Catalog Object Model</v>
+        <v>Partitioning on Databricks</v>
       </c>
       <c r="C42" s="2" t="str">
         <f>'Databricks Master Syllabus'!A38</f>
-        <v>6. Unity Catalog &amp; Governance</v>
+        <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
@@ -4595,14 +5036,14 @@
       </c>
       <c r="B43" s="3" t="str">
         <f>'Databricks Master Syllabus'!C39</f>
-        <v>Managed vs External Tables</v>
+        <v>Unity Catalog Object Model</v>
       </c>
       <c r="C43" s="3" t="str">
         <f>'Databricks Master Syllabus'!A39</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E43" s="3">
         <v>0</v>
@@ -4617,14 +5058,14 @@
       </c>
       <c r="B44" s="2" t="str">
         <f>'Databricks Master Syllabus'!C40</f>
-        <v>Volumes</v>
+        <v>Managed vs External Tables</v>
       </c>
       <c r="C44" s="2" t="str">
         <f>'Databricks Master Syllabus'!A40</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E44" s="2">
         <v>0</v>
@@ -4633,20 +5074,20 @@
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>40</v>
       </c>
       <c r="B45" s="3" t="str">
         <f>'Databricks Master Syllabus'!C41</f>
-        <v>Storage Credentials and External Locations on Azure</v>
+        <v>Volumes</v>
       </c>
       <c r="C45" s="3" t="str">
         <f>'Databricks Master Syllabus'!A41</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E45" s="3">
         <v>0</v>
@@ -4655,20 +5096,20 @@
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>41</v>
       </c>
       <c r="B46" s="2" t="str">
         <f>'Databricks Master Syllabus'!C42</f>
-        <v>Privileges and Inheritance</v>
+        <v>Storage Credentials and External Locations on Azure</v>
       </c>
       <c r="C46" s="2" t="str">
         <f>'Databricks Master Syllabus'!A42</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E46" s="2">
         <v>0</v>
@@ -4683,14 +5124,14 @@
       </c>
       <c r="B47" s="3" t="str">
         <f>'Databricks Master Syllabus'!C43</f>
-        <v>Ownership and the Missing DENY</v>
+        <v>Privileges and Inheritance</v>
       </c>
       <c r="C47" s="3" t="str">
         <f>'Databricks Master Syllabus'!A43</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E47" s="3">
         <v>0</v>
@@ -4705,14 +5146,14 @@
       </c>
       <c r="B48" s="2" t="str">
         <f>'Databricks Master Syllabus'!C44</f>
-        <v>Row Filters and Column Masks</v>
+        <v>Ownership and the Missing DENY</v>
       </c>
       <c r="C48" s="2" t="str">
         <f>'Databricks Master Syllabus'!A44</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E48" s="2">
         <v>0</v>
@@ -4727,14 +5168,14 @@
       </c>
       <c r="B49" s="3" t="str">
         <f>'Databricks Master Syllabus'!C45</f>
-        <v>ABAC and Dynamic Views</v>
+        <v>Row Filters and Column Masks</v>
       </c>
       <c r="C49" s="3" t="str">
         <f>'Databricks Master Syllabus'!A45</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E49" s="3">
         <v>0</v>
@@ -4749,14 +5190,14 @@
       </c>
       <c r="B50" s="2" t="str">
         <f>'Databricks Master Syllabus'!C46</f>
-        <v>Lineage and Audit</v>
+        <v>ABAC and Dynamic Views</v>
       </c>
       <c r="C50" s="2" t="str">
         <f>'Databricks Master Syllabus'!A46</f>
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E50" s="2">
         <v>0</v>
@@ -4771,14 +5212,14 @@
       </c>
       <c r="B51" s="3" t="str">
         <f>'Databricks Master Syllabus'!C47</f>
-        <v>Serverless vs Classic Compute</v>
+        <v>Lineage and Audit</v>
       </c>
       <c r="C51" s="3" t="str">
         <f>'Databricks Master Syllabus'!A47</f>
-        <v>7. Compute &amp; Cost</v>
+        <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E51" s="3">
         <v>0</v>
@@ -4793,14 +5234,14 @@
       </c>
       <c r="B52" s="2" t="str">
         <f>'Databricks Master Syllabus'!C48</f>
-        <v>All-Purpose vs Job Compute</v>
+        <v>Serverless vs Classic Compute</v>
       </c>
       <c r="C52" s="2" t="str">
         <f>'Databricks Master Syllabus'!A48</f>
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E52" s="2">
         <v>0</v>
@@ -4815,14 +5256,14 @@
       </c>
       <c r="B53" s="3" t="str">
         <f>'Databricks Master Syllabus'!C49</f>
-        <v>SQL Warehouses</v>
+        <v>All-Purpose vs Job Compute</v>
       </c>
       <c r="C53" s="3" t="str">
         <f>'Databricks Master Syllabus'!A49</f>
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E53" s="3">
         <v>0</v>
@@ -4837,14 +5278,14 @@
       </c>
       <c r="B54" s="2" t="str">
         <f>'Databricks Master Syllabus'!C50</f>
-        <v>Access Modes</v>
+        <v>SQL Warehouses</v>
       </c>
       <c r="C54" s="2" t="str">
         <f>'Databricks Master Syllabus'!A50</f>
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E54" s="2">
         <v>0</v>
@@ -4859,14 +5300,14 @@
       </c>
       <c r="B55" s="3" t="str">
         <f>'Databricks Master Syllabus'!C51</f>
-        <v>Compute Policies and Pools</v>
+        <v>Access Modes</v>
       </c>
       <c r="C55" s="3" t="str">
         <f>'Databricks Master Syllabus'!A51</f>
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E55" s="3">
         <v>0</v>
@@ -4881,14 +5322,14 @@
       </c>
       <c r="B56" s="2" t="str">
         <f>'Databricks Master Syllabus'!C52</f>
-        <v>DBUs and Cost Levers</v>
+        <v>Photon and Runtime Selection</v>
       </c>
       <c r="C56" s="2" t="str">
         <f>'Databricks Master Syllabus'!A52</f>
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E56" s="2">
         <v>0</v>
@@ -4897,20 +5338,20 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A57" s="3">
         <v>52</v>
       </c>
       <c r="B57" s="3" t="str">
         <f>'Databricks Master Syllabus'!C53</f>
-        <v>Spark Execution Model</v>
+        <v>Compute Policies, Pools and Autoscaling</v>
       </c>
       <c r="C57" s="3" t="str">
         <f>'Databricks Master Syllabus'!A53</f>
-        <v>8. Spark &amp; Transformation</v>
+        <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E57" s="3">
         <v>0</v>
@@ -4919,20 +5360,20 @@
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
     </row>
-    <row r="58" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>53</v>
       </c>
       <c r="B58" s="2" t="str">
         <f>'Databricks Master Syllabus'!C54</f>
-        <v>DataFrame and SQL Transformations</v>
+        <v>DBUs and Cost Levers</v>
       </c>
       <c r="C58" s="2" t="str">
         <f>'Databricks Master Syllabus'!A54</f>
-        <v>8. Spark &amp; Transformation</v>
+        <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E58" s="2">
         <v>0</v>
@@ -4947,14 +5388,14 @@
       </c>
       <c r="B59" s="3" t="str">
         <f>'Databricks Master Syllabus'!C55</f>
-        <v>Joins, Unions and Deduplication</v>
+        <v>Spark Execution Model</v>
       </c>
       <c r="C59" s="3" t="str">
         <f>'Databricks Master Syllabus'!A55</f>
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E59" s="3">
         <v>0</v>
@@ -4963,20 +5404,20 @@
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>55</v>
       </c>
       <c r="B60" s="2" t="str">
         <f>'Databricks Master Syllabus'!C56</f>
-        <v>Bronze to Silver to Gold</v>
+        <v>DataFrame and SQL Transformations</v>
       </c>
       <c r="C60" s="2" t="str">
         <f>'Databricks Master Syllabus'!A56</f>
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E60" s="2">
         <v>0</v>
@@ -4985,20 +5426,20 @@
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="3">
         <v>56</v>
       </c>
       <c r="B61" s="3" t="str">
         <f>'Databricks Master Syllabus'!C57</f>
-        <v>AQE, Broadcast and Shuffle Partitions</v>
+        <v>Joins, Unions and Deduplication</v>
       </c>
       <c r="C61" s="3" t="str">
         <f>'Databricks Master Syllabus'!A57</f>
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E61" s="3">
         <v>0</v>
@@ -5013,14 +5454,14 @@
       </c>
       <c r="B62" s="2" t="str">
         <f>'Databricks Master Syllabus'!C58</f>
-        <v>Skew, Salting and Spill</v>
+        <v>Bronze to Silver to Gold</v>
       </c>
       <c r="C62" s="2" t="str">
         <f>'Databricks Master Syllabus'!A58</f>
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E62" s="2">
         <v>0</v>
@@ -5029,20 +5470,20 @@
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A63" s="3">
         <v>58</v>
       </c>
       <c r="B63" s="3" t="str">
         <f>'Databricks Master Syllabus'!C59</f>
-        <v>Disk Cache and the Spark UI</v>
+        <v>AQE, Broadcast and Shuffle Partitions</v>
       </c>
       <c r="C63" s="3" t="str">
         <f>'Databricks Master Syllabus'!A59</f>
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E63" s="3">
         <v>0</v>
@@ -5057,14 +5498,14 @@
       </c>
       <c r="B64" s="2" t="str">
         <f>'Databricks Master Syllabus'!C60</f>
-        <v>Choosing an Ingestion Method</v>
+        <v>Skew, Salting and Spill</v>
       </c>
       <c r="C64" s="2" t="str">
         <f>'Databricks Master Syllabus'!A60</f>
-        <v>9. Ingestion &amp; Streaming</v>
+        <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E64" s="2">
         <v>0</v>
@@ -5079,14 +5520,14 @@
       </c>
       <c r="B65" s="3" t="str">
         <f>'Databricks Master Syllabus'!C61</f>
-        <v>COPY INTO</v>
+        <v>Disk Cache and the Spark UI</v>
       </c>
       <c r="C65" s="3" t="str">
         <f>'Databricks Master Syllabus'!A61</f>
-        <v>9. Ingestion &amp; Streaming</v>
+        <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E65" s="3">
         <v>0</v>
@@ -5101,14 +5542,14 @@
       </c>
       <c r="B66" s="2" t="str">
         <f>'Databricks Master Syllabus'!C62</f>
-        <v>Auto Loader File Detection</v>
+        <v>Choosing an Ingestion Method</v>
       </c>
       <c r="C66" s="2" t="str">
         <f>'Databricks Master Syllabus'!A62</f>
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E66" s="2">
         <v>0</v>
@@ -5117,20 +5558,20 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="3">
         <v>62</v>
       </c>
       <c r="B67" s="3" t="str">
         <f>'Databricks Master Syllabus'!C63</f>
-        <v>Auto Loader Schema Inference and Evolution</v>
+        <v>COPY INTO</v>
       </c>
       <c r="C67" s="3" t="str">
         <f>'Databricks Master Syllabus'!A63</f>
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E67" s="3">
         <v>0</v>
@@ -5145,14 +5586,14 @@
       </c>
       <c r="B68" s="2" t="str">
         <f>'Databricks Master Syllabus'!C64</f>
-        <v>Structured Streaming Checkpoints</v>
+        <v>Auto Loader File Detection</v>
       </c>
       <c r="C68" s="2" t="str">
         <f>'Databricks Master Syllabus'!A64</f>
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E68" s="2">
         <v>0</v>
@@ -5167,14 +5608,14 @@
       </c>
       <c r="B69" s="3" t="str">
         <f>'Databricks Master Syllabus'!C65</f>
-        <v>Triggers, Watermarks and Output Modes</v>
+        <v>Auto Loader Schema Inference and Evolution</v>
       </c>
       <c r="C69" s="3" t="str">
         <f>'Databricks Master Syllabus'!A65</f>
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E69" s="3">
         <v>0</v>
@@ -5189,14 +5630,14 @@
       </c>
       <c r="B70" s="2" t="str">
         <f>'Databricks Master Syllabus'!C66</f>
-        <v>foreachBatch and Exactly-Once</v>
+        <v>Structured Streaming Checkpoints</v>
       </c>
       <c r="C70" s="2" t="str">
         <f>'Databricks Master Syllabus'!A66</f>
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E70" s="2">
         <v>0</v>
@@ -5211,14 +5652,14 @@
       </c>
       <c r="B71" s="3" t="str">
         <f>'Databricks Master Syllabus'!C67</f>
-        <v>Streaming Tables vs Materialized Views</v>
+        <v>Triggers, Watermarks and Output Modes</v>
       </c>
       <c r="C71" s="3" t="str">
         <f>'Databricks Master Syllabus'!A67</f>
-        <v>10. Pipelines &amp; Orchestration</v>
+        <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E71" s="3">
         <v>0</v>
@@ -5233,14 +5674,14 @@
       </c>
       <c r="B72" s="2" t="str">
         <f>'Databricks Master Syllabus'!C68</f>
-        <v>Expectations</v>
+        <v>foreachBatch and Exactly-Once</v>
       </c>
       <c r="C72" s="2" t="str">
         <f>'Databricks Master Syllabus'!A68</f>
-        <v>10. Pipelines &amp; Orchestration</v>
+        <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E72" s="2">
         <v>0</v>
@@ -5255,14 +5696,14 @@
       </c>
       <c r="B73" s="3" t="str">
         <f>'Databricks Master Syllabus'!C69</f>
-        <v>AUTO CDC and SCD Types</v>
+        <v>Recovery, Replay and Backfill</v>
       </c>
       <c r="C73" s="3" t="str">
         <f>'Databricks Master Syllabus'!A69</f>
-        <v>10. Pipelines &amp; Orchestration</v>
+        <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E73" s="3">
         <v>0</v>
@@ -5277,14 +5718,14 @@
       </c>
       <c r="B74" s="2" t="str">
         <f>'Databricks Master Syllabus'!C70</f>
-        <v>Refresh vs Full Refresh</v>
+        <v>Pipeline Datasets and Flows</v>
       </c>
       <c r="C74" s="2" t="str">
         <f>'Databricks Master Syllabus'!A70</f>
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E74" s="2">
         <v>0</v>
@@ -5293,20 +5734,20 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="3">
         <v>70</v>
       </c>
       <c r="B75" s="3" t="str">
         <f>'Databricks Master Syllabus'!C71</f>
-        <v>Lakeflow Jobs: Tasks and Dependencies</v>
+        <v>Expectations</v>
       </c>
       <c r="C75" s="3" t="str">
         <f>'Databricks Master Syllabus'!A71</f>
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E75" s="3">
         <v>0</v>
@@ -5321,14 +5762,14 @@
       </c>
       <c r="B76" s="2" t="str">
         <f>'Databricks Master Syllabus'!C72</f>
-        <v>Run If, Retries and Timeouts</v>
+        <v>AUTO CDC and SCD Types</v>
       </c>
       <c r="C76" s="2" t="str">
         <f>'Databricks Master Syllabus'!A72</f>
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E76" s="2">
         <v>0</v>
@@ -5343,14 +5784,14 @@
       </c>
       <c r="B77" s="3" t="str">
         <f>'Databricks Master Syllabus'!C73</f>
-        <v>Triggers and Repair Runs</v>
+        <v>Refresh vs Full Refresh</v>
       </c>
       <c r="C77" s="3" t="str">
         <f>'Databricks Master Syllabus'!A73</f>
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E77" s="3">
         <v>0</v>
@@ -5359,20 +5800,20 @@
       <c r="G77" s="3"/>
       <c r="H77" s="3"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>73</v>
       </c>
       <c r="B78" s="2" t="str">
         <f>'Databricks Master Syllabus'!C74</f>
-        <v>Databricks with ADF and ADLS</v>
+        <v>Lakeflow Jobs: Tasks and Dependencies</v>
       </c>
       <c r="C78" s="2" t="str">
         <f>'Databricks Master Syllabus'!A74</f>
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E78" s="2">
         <v>0</v>
@@ -5387,14 +5828,14 @@
       </c>
       <c r="B79" s="3" t="str">
         <f>'Databricks Master Syllabus'!C75</f>
-        <v>System Tables and Monitoring</v>
+        <v>Run If, Retries and Timeouts</v>
       </c>
       <c r="C79" s="3" t="str">
         <f>'Databricks Master Syllabus'!A75</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E79" s="3">
         <v>0</v>
@@ -5403,20 +5844,20 @@
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
     </row>
-    <row r="80" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>75</v>
       </c>
       <c r="B80" s="2" t="str">
         <f>'Databricks Master Syllabus'!C76</f>
-        <v>Pipeline Event Logs and Job Run History</v>
+        <v>Job Concurrency and Limits</v>
       </c>
       <c r="C80" s="2" t="str">
         <f>'Databricks Master Syllabus'!A76</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E80" s="2">
         <v>0</v>
@@ -5431,14 +5872,14 @@
       </c>
       <c r="B81" s="3" t="str">
         <f>'Databricks Master Syllabus'!C77</f>
-        <v>Identity and Secrets</v>
+        <v>Triggers and Repair Runs</v>
       </c>
       <c r="C81" s="3" t="str">
         <f>'Databricks Master Syllabus'!A77</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E81" s="3">
         <v>0</v>
@@ -5453,14 +5894,14 @@
       </c>
       <c r="B82" s="2" t="str">
         <f>'Databricks Master Syllabus'!C78</f>
-        <v>Git Folders</v>
+        <v>Databricks with ADF and ADLS</v>
       </c>
       <c r="C82" s="2" t="str">
         <f>'Databricks Master Syllabus'!A78</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E82" s="2">
         <v>0</v>
@@ -5475,14 +5916,14 @@
       </c>
       <c r="B83" s="3" t="str">
         <f>'Databricks Master Syllabus'!C79</f>
-        <v>Declarative Automation Bundles</v>
+        <v>Three Network Connections</v>
       </c>
       <c r="C83" s="3" t="str">
         <f>'Databricks Master Syllabus'!A79</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E83" s="3">
         <v>0</v>
@@ -5491,20 +5932,20 @@
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
     </row>
-    <row r="84" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>79</v>
       </c>
       <c r="B84" s="2" t="str">
         <f>'Databricks Master Syllabus'!C80</f>
-        <v>Capstone: End-to-End Medallion Pipeline</v>
+        <v>Serverless vs Hybrid Workspaces</v>
       </c>
       <c r="C84" s="2" t="str">
         <f>'Databricks Master Syllabus'!A80</f>
-        <v>11. Operate, Deploy &amp; Capstone</v>
+        <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="E84" s="2">
         <v>0</v>
@@ -5512,6 +5953,270 @@
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A85" s="3">
+        <v>80</v>
+      </c>
+      <c r="B85" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C81</f>
+        <v>VNet Injection and Subnet Sizing</v>
+      </c>
+      <c r="C85" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A81</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E85" s="3">
+        <v>0</v>
+      </c>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A86" s="2">
+        <v>81</v>
+      </c>
+      <c r="B86" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C82</f>
+        <v>Subnet Delegation and NSG Rules</v>
+      </c>
+      <c r="C86" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A82</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E86" s="2">
+        <v>0</v>
+      </c>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+    </row>
+    <row r="87" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A87" s="3">
+        <v>82</v>
+      </c>
+      <c r="B87" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C83</f>
+        <v>Secure Cluster Connectivity and Egress</v>
+      </c>
+      <c r="C87" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A83</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E87" s="3">
+        <v>0</v>
+      </c>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A88" s="2">
+        <v>83</v>
+      </c>
+      <c r="B88" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C84</f>
+        <v>Private Link: Three Kinds</v>
+      </c>
+      <c r="C88" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A84</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E88" s="2">
+        <v>0</v>
+      </c>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+    </row>
+    <row r="89" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A89" s="3">
+        <v>84</v>
+      </c>
+      <c r="B89" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C85</f>
+        <v>Browser Authentication and the Transit VNet</v>
+      </c>
+      <c r="C89" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A85</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E89" s="3">
+        <v>0</v>
+      </c>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+    </row>
+    <row r="90" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A90" s="2">
+        <v>85</v>
+      </c>
+      <c r="B90" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C86</f>
+        <v>Serverless Connectivity and Storage Firewalls</v>
+      </c>
+      <c r="C90" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A86</f>
+        <v>11. Azure Networking for Databricks</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E90" s="2">
+        <v>0</v>
+      </c>
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+      <c r="H90" s="2"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A91" s="3">
+        <v>86</v>
+      </c>
+      <c r="B91" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C87</f>
+        <v>System Tables and Monitoring</v>
+      </c>
+      <c r="C91" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A87</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E91" s="3">
+        <v>0</v>
+      </c>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+    </row>
+    <row r="92" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A92" s="2">
+        <v>87</v>
+      </c>
+      <c r="B92" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C88</f>
+        <v>Pipeline Event Logs and Job Run History</v>
+      </c>
+      <c r="C92" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A88</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E92" s="2">
+        <v>0</v>
+      </c>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A93" s="3">
+        <v>88</v>
+      </c>
+      <c r="B93" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C89</f>
+        <v>Identity and Secrets</v>
+      </c>
+      <c r="C93" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A89</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E93" s="3">
+        <v>0</v>
+      </c>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A94" s="2">
+        <v>89</v>
+      </c>
+      <c r="B94" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C90</f>
+        <v>Git Folders</v>
+      </c>
+      <c r="C94" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A90</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E94" s="2">
+        <v>0</v>
+      </c>
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
+      <c r="H94" s="2"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A95" s="3">
+        <v>90</v>
+      </c>
+      <c r="B95" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C91</f>
+        <v>Declarative Automation Bundles</v>
+      </c>
+      <c r="C95" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A91</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E95" s="3">
+        <v>0</v>
+      </c>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+    </row>
+    <row r="96" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A96" s="2">
+        <v>91</v>
+      </c>
+      <c r="B96" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C92</f>
+        <v>Capstone: End-to-End Medallion Pipeline</v>
+      </c>
+      <c r="C96" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A92</f>
+        <v>12. Operate, Deploy &amp; Capstone</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E96" s="2">
+        <v>0</v>
+      </c>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
+      <c r="H96" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5530,178 +6235,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>317</v>
+        <v>360</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>318</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>319</v>
+        <v>362</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>320</v>
+        <v>363</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>321</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>322</v>
+        <v>365</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>323</v>
+        <v>366</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>324</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>325</v>
+        <v>368</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>326</v>
+        <v>369</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>327</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>328</v>
+        <v>371</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>329</v>
+        <v>372</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>331</v>
+        <v>374</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>332</v>
+        <v>375</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>333</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>334</v>
+        <v>377</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>335</v>
+        <v>378</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>333</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>336</v>
+        <v>379</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>337</v>
+        <v>380</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>333</v>
+        <v>376</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>338</v>
+        <v>381</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>339</v>
+        <v>382</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>340</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>341</v>
+        <v>384</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>342</v>
+        <v>385</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>343</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>344</v>
+        <v>387</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>345</v>
+        <v>388</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>346</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>347</v>
+        <v>390</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>348</v>
+        <v>391</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>349</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>350</v>
+        <v>393</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>351</v>
+        <v>394</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>349</v>
+        <v>392</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>352</v>
+        <v>395</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>353</v>
+        <v>396</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>354</v>
+        <v>397</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>355</v>
+        <v>398</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>356</v>
+        <v>399</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>333</v>
+        <v>376</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>357</v>
+        <v>400</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>358</v>
+        <v>401</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>359</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -5720,130 +6425,130 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>360</v>
+        <v>403</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>361</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>363</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>364</v>
+        <v>407</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>365</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>368</v>
+        <v>411</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>369</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>370</v>
+        <v>413</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>371</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>372</v>
+        <v>415</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>373</v>
+        <v>416</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>374</v>
+        <v>417</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>375</v>
+        <v>418</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>376</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>328</v>
+        <v>371</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>377</v>
+        <v>420</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>378</v>
+        <v>421</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>379</v>
+        <v>422</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>380</v>
+        <v>423</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>381</v>
+        <v>424</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>382</v>
+        <v>425</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>383</v>
+        <v>426</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>384</v>
+        <v>427</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>385</v>
+        <v>428</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>386</v>
+        <v>429</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>387</v>
+        <v>430</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>388</v>
+        <v>431</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>389</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add production, troubleshooting and an error catalogue to the Databricks roadmap
Notes gain section 23 (streams in production, stateful streaming,
notifications and SQL alerts, failed-job troubleshooting, error conditions,
query profile, compute start-up failures, libraries and init scripts,
runtime lifecycle, environment isolation, encryption keys, HA and DR,
testing) and section 24, an error catalogue taken from the official
error-conditions reference. Section 19 records that two pages disagree on
default task retries. The roadmap gains phase 13 (17 topics) and an Error
Catalogue sheet of 35 rows; 108 topics in 13 phases. All five sheets pass
the import preview on a scratch database.
</commit_message>
<xml_diff>
--- a/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
+++ b/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\PrepBench\.claude\worktrees\databricks-research-1e243f\docs\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34323425-181B-4317-BD98-F283F90A0AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4230A312-1C88-4DD3-BD53-B23662758D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Journey Progress Tracker" sheetId="2" r:id="rId2"/>
     <sheet name="Databricks Command Reference" sheetId="3" r:id="rId3"/>
     <sheet name="Mental Model" sheetId="4" r:id="rId4"/>
+    <sheet name="Error Catalogue" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="640">
   <si>
     <t>Phase</t>
   </si>
@@ -881,7 +882,7 @@
     <t>Run If, Retries and Timeouts</t>
   </si>
   <si>
-    <t>Master Run if conditions, retry policies (none by default), and timeouts.</t>
+    <t>Master Run if conditions, retry policies (set them explicitly), and timeouts.</t>
   </si>
   <si>
     <t>Configure a cleanup task that runs even when an upstream task fails, and a retry on a flaky task.</t>
@@ -1004,7 +1005,7 @@
     <t>Diagnose a serverless job getting 403 Forbidden from a firewalled ADLS account and give the fix.</t>
   </si>
   <si>
-    <t>12. Operate, Deploy &amp; Capstone</t>
+    <t>12. Operate &amp; Deploy</t>
   </si>
   <si>
     <t>System Tables and Monitoring</t>
@@ -1064,6 +1065,213 @@
     <t>Deploy one job to dev and prod targets with a different schema name per target.</t>
   </si>
   <si>
+    <t>13. Production, Troubleshooting &amp; Capstone</t>
+  </si>
+  <si>
+    <t>Running Streams in Production</t>
+  </si>
+  <si>
+    <t>Master production streaming: jobs compute, Continuous job mode, no autoscaling, automatic restart with backoff, no awaitTermination, one job per critical stream.</t>
+  </si>
+  <si>
+    <t>Review a streaming job's settings and list every change needed before it goes to production.</t>
+  </si>
+  <si>
+    <t>§23.1</t>
+  </si>
+  <si>
+    <t>Stateful Streaming in Production</t>
+  </si>
+  <si>
+    <t>Understand state (aggregations, dropDuplicates, stream joins), RocksDB with changelog checkpointing, and shuffle partitions fixed when the checkpoint is created.</t>
+  </si>
+  <si>
+    <t>Explain why raising spark.sql.shuffle.partitions didn't change a running stateful query, and what would.</t>
+  </si>
+  <si>
+    <t>§23.2</t>
+  </si>
+  <si>
+    <t>Notifications and Alerts</t>
+  </si>
+  <si>
+    <t>Master job and task notifications (failure, duration, streaming backlog), destinations, and Databricks SQL alerts on a query result.</t>
+  </si>
+  <si>
+    <t>Set up notifications so a failing task in a multi-task streaming job is noticed within minutes.</t>
+  </si>
+  <si>
+    <t>§23.3</t>
+  </si>
+  <si>
+    <t>Troubleshooting a Failed Job</t>
+  </si>
+  <si>
+    <t>Master the path from alert to cause: Runs tab, matrix view, task run details, common causes, repair with current settings, continuous-job backoff.</t>
+  </si>
+  <si>
+    <t>Walk through a failed run step by step and decide whether repairing it is safe.</t>
+  </si>
+  <si>
+    <t>§23.4</t>
+  </si>
+  <si>
+    <t>Reading Errors: Conditions and SQLSTATE</t>
+  </si>
+  <si>
+    <t>Understand error conditions, SQLSTATE and message parameters, and why code should match the condition, never the message text.</t>
+  </si>
+  <si>
+    <t>Catch TABLE_OR_VIEW_NOT_FOUND in Python by its condition and print its SQLSTATE in Free Edition.</t>
+  </si>
+  <si>
+    <t>§23.5</t>
+  </si>
+  <si>
+    <t>Write, Schema and MERGE Errors</t>
+  </si>
+  <si>
+    <t>Diagnose column-count mismatches, failed schema merges, incompatible types, duplicate MERGE source rows and append-only tables.</t>
+  </si>
+  <si>
+    <t>Reproduce DELTA_MULTIPLE_SOURCE_ROW_MATCHING_TARGET_ROW_IN_MERGE in Free Edition and fix it.</t>
+  </si>
+  <si>
+    <t>§24.2</t>
+  </si>
+  <si>
+    <t>Concurrent Write Conflicts</t>
+  </si>
+  <si>
+    <t>Diagnose the DELTA_CONCURRENT_* family, metadata and protocol changes, and two streams sharing one checkpoint.</t>
+  </si>
+  <si>
+    <t>Name the likely cause and fix for each of five concurrent-write errors.</t>
+  </si>
+  <si>
+    <t>§24.3, §2.7</t>
+  </si>
+  <si>
+    <t>Streaming Errors</t>
+  </si>
+  <si>
+    <t>Diagnose new-field failures, missing notified files, schema changes under a stream, update/delete commits in a streamed table, and out-of-memory on restart.</t>
+  </si>
+  <si>
+    <t>For each streaming error, say whether a restart, a new checkpoint, an option or more compute is the fix.</t>
+  </si>
+  <si>
+    <t>§24.4, §23.1</t>
+  </si>
+  <si>
+    <t>File, History and Retention Errors</t>
+  </si>
+  <si>
+    <t>Diagnose missing files referenced by the log, VACUUM retention and LITE errors, time travel past retention, and unsupported table features.</t>
+  </si>
+  <si>
+    <t>Explain how a too-short VACUUM retention turned into DELTA_FILE_NOT_FOUND_DETAILED for a stream.</t>
+  </si>
+  <si>
+    <t>§24.5</t>
+  </si>
+  <si>
+    <t>Query Profile and Query History</t>
+  </si>
+  <si>
+    <t>Use query history and the query profile to find the slowest operators, exploding joins and full scans.</t>
+  </si>
+  <si>
+    <t>In Free Edition, open a slow query's profile and name its most expensive operator.</t>
+  </si>
+  <si>
+    <t>§23.6</t>
+  </si>
+  <si>
+    <t>Compute That Won't Start</t>
+  </si>
+  <si>
+    <t>Understand the 'compute plane network is misconfigured' and METASTORE_DOWN symptoms and how to test the network path on Azure.</t>
+  </si>
+  <si>
+    <t>List the endpoints you would test from a VM in the workspace subnet, and why.</t>
+  </si>
+  <si>
+    <t>§23.7, §20</t>
+  </si>
+  <si>
+    <t>Libraries and Init Scripts</t>
+  </si>
+  <si>
+    <t>Understand compute-scoped libraries from volumes, why DBFS libraries are discouraged, and Databricks' advice to avoid init scripts (none on serverless).</t>
+  </si>
+  <si>
+    <t>Move a library install out of an init script into a compute policy and explain the gain.</t>
+  </si>
+  <si>
+    <t>§23.8</t>
+  </si>
+  <si>
+    <t>Runtime Lifecycle and Upgrades</t>
+  </si>
+  <si>
+    <t>Understand the runtime lifecycle (six months of features, LTS fixes for three years, end of support) and feature retirement phases.</t>
+  </si>
+  <si>
+    <t>Plan when a team on an LTS runtime must upgrade and what to test first.</t>
+  </si>
+  <si>
+    <t>§23.9</t>
+  </si>
+  <si>
+    <t>Environment Isolation and Catalog Strategy</t>
+  </si>
+  <si>
+    <t>Understand separate workspaces for environments or business units, their costs, and catalogs as data domains with separate storage.</t>
+  </si>
+  <si>
+    <t>Propose a dev/test/prod layout of workspaces and catalogs and name one trade-off.</t>
+  </si>
+  <si>
+    <t>§23.10</t>
+  </si>
+  <si>
+    <t>Encryption and Customer-Managed Keys</t>
+  </si>
+  <si>
+    <t>Understand Azure customer-managed keys for managed disks, managed services and the DBFS root, and that traffic between workers isn't encrypted by default.</t>
+  </si>
+  <si>
+    <t>Say which key protects notebook source, cluster temp disks and the workspace storage account.</t>
+  </si>
+  <si>
+    <t>§23.11</t>
+  </si>
+  <si>
+    <t>High Availability and Disaster Recovery</t>
+  </si>
+  <si>
+    <t>Understand zone-level HA vs cross-region DR, RPO and RTO, active-passive, managed DR, Deep Clone replication, and why DR doesn't fix corruption.</t>
+  </si>
+  <si>
+    <t>Explain to a sponsor why a DR region didn't help when a bad job corrupted a table, and what would have.</t>
+  </si>
+  <si>
+    <t>§23.12</t>
+  </si>
+  <si>
+    <t>Testing Databricks Code</t>
+  </si>
+  <si>
+    <t>Understand unit testing functions with pytest and SQL UDFs, kept outside notebooks in a Git folder.</t>
+  </si>
+  <si>
+    <t>Write one pytest test for a transformation function and run it from a Git folder.</t>
+  </si>
+  <si>
+    <t>§23.13</t>
+  </si>
+  <si>
     <t>Capstone: End-to-End Medallion Pipeline</t>
   </si>
   <si>
@@ -1073,7 +1281,7 @@
     <t>Run the pipeline in Free Edition, grant a reader group on gold, and explain every design choice to a reviewer.</t>
   </si>
   <si>
-    <t>1-23</t>
+    <t>1-24</t>
   </si>
   <si>
     <t>all</t>
@@ -1335,6 +1543,420 @@
   </si>
   <si>
     <t>Ore, refined metal, finished jewellery: each stage is cleaner and closer to what the customer wants.</t>
+  </si>
+  <si>
+    <t>Error Condition (SQLSTATE)</t>
+  </si>
+  <si>
+    <t>What You See</t>
+  </si>
+  <si>
+    <t>Likely Cause and Fix</t>
+  </si>
+  <si>
+    <t>Taught In (#)</t>
+  </si>
+  <si>
+    <t>TABLE_OR_VIEW_NOT_FOUND (42P01)</t>
+  </si>
+  <si>
+    <t>The table or view can't be found</t>
+  </si>
+  <si>
+    <t>Wrong name, wrong current schema, or no USE CATALOG/USE SCHEMA. Fix: Qualify catalog.schema.table; check grants.</t>
+  </si>
+  <si>
+    <t>38, 95</t>
+  </si>
+  <si>
+    <t>SCHEMA_NOT_FOUND (42704)</t>
+  </si>
+  <si>
+    <t>The schema can't be found</t>
+  </si>
+  <si>
+    <t>Wrong name or catalog. Fix: Qualify the name with its catalog.</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>UNRESOLVED_COLUMN (42703)</t>
+  </si>
+  <si>
+    <t>A column or parameter can't be resolved</t>
+  </si>
+  <si>
+    <t>Misspelt or missing column. Fix: Check the DataFrame's columns.</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>INSUFFICIENT_PERMISSIONS (42501)</t>
+  </si>
+  <si>
+    <t>Insufficient privileges</t>
+  </si>
+  <si>
+    <t>A missing privilege in the USE CATALOG + USE SCHEMA + object chain. Fix: Grant the missing privilege.</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>INSUFFICIENT_PERMISSIONS_EXT_LOC (42501)</t>
+  </si>
+  <si>
+    <t>Insufficient privileges on an external location</t>
+  </si>
+  <si>
+    <t>No privilege on the external location. Fix: Grant it on the external location.</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>CAST_INVALID_INPUT (22018)</t>
+  </si>
+  <si>
+    <t>A malformed value can't be cast</t>
+  </si>
+  <si>
+    <t>Bad source data. Fix: Fix the data or type; try_cast returns NULL.</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>DIVIDE_BY_ZERO (22012)</t>
+  </si>
+  <si>
+    <t>Division by zero</t>
+  </si>
+  <si>
+    <t>A zero divisor. Fix: try_divide returns NULL.</t>
+  </si>
+  <si>
+    <t>DELTA_INSERT_COLUMN_ARITY_MISMATCH (42802)</t>
+  </si>
+  <si>
+    <t>Target has N columns, the data has M</t>
+  </si>
+  <si>
+    <t>Source and table schemas differ. Fix: Align columns or evolve the schema on purpose.</t>
+  </si>
+  <si>
+    <t>27, 96</t>
+  </si>
+  <si>
+    <t>DELTA_FAILED_TO_MERGE_FIELDS (22005)</t>
+  </si>
+  <si>
+    <t>Two field definitions can't be merged</t>
+  </si>
+  <si>
+    <t>Type conflict during schema merge. Fix: Cast the source or change the table.</t>
+  </si>
+  <si>
+    <t>28, 96</t>
+  </si>
+  <si>
+    <t>DELTA_MERGE_INCOMPATIBLE_DATATYPE (42K09)</t>
+  </si>
+  <si>
+    <t>Incompatible data types can't be merged</t>
+  </si>
+  <si>
+    <t>Type conflict. Fix: Cast the source or change the table.</t>
+  </si>
+  <si>
+    <t>DELTA_MULTIPLE_SOURCE_ROW_MATCHING_TARGET_ROW_IN_MERGE (21506)</t>
+  </si>
+  <si>
+    <t>Several source rows match one target row</t>
+  </si>
+  <si>
+    <t>Duplicate keys in the MERGE source. Fix: Deduplicate the source first.</t>
+  </si>
+  <si>
+    <t>29, 96</t>
+  </si>
+  <si>
+    <t>DELTA_CANNOT_MODIFY_APPEND_ONLY (42809)</t>
+  </si>
+  <si>
+    <t>The table only allows appends</t>
+  </si>
+  <si>
+    <t>Table property set to append-only. Fix: Change it only if updates are really allowed.</t>
+  </si>
+  <si>
+    <t>96</t>
+  </si>
+  <si>
+    <t>DELTA_CONCURRENT_APPEND (2D521)</t>
+  </si>
+  <si>
+    <t>A concurrent operation added conflicting data</t>
+  </si>
+  <si>
+    <t>Two writers overlapping. Fix: Retry; reduce overlap.</t>
+  </si>
+  <si>
+    <t>18, 97</t>
+  </si>
+  <si>
+    <t>DELTA_CONCURRENT_DELETE_READ (2D521)</t>
+  </si>
+  <si>
+    <t>Data this transaction read was deleted concurrently</t>
+  </si>
+  <si>
+    <t>An overlapping delete. Fix: Retry.</t>
+  </si>
+  <si>
+    <t>DELTA_CONCURRENT_WRITE (2D521)</t>
+  </si>
+  <si>
+    <t>New data was written since this transaction read</t>
+  </si>
+  <si>
+    <t>A concurrent write. Fix: Try the operation again.</t>
+  </si>
+  <si>
+    <t>DELTA_CONCURRENT_TRANSACTION (2D521)</t>
+  </si>
+  <si>
+    <t>Several streams use the same checkpoint</t>
+  </si>
+  <si>
+    <t>A duplicate run of one streaming query. Fix: One checkpoint per query; stop the duplicate.</t>
+  </si>
+  <si>
+    <t>65, 97</t>
+  </si>
+  <si>
+    <t>DELTA_METADATA_CHANGED (2D521)</t>
+  </si>
+  <si>
+    <t>Metadata changed by a concurrent update</t>
+  </si>
+  <si>
+    <t>A schema or property change during writes. Fix: Retry; schedule changes away from writes.</t>
+  </si>
+  <si>
+    <t>19, 97</t>
+  </si>
+  <si>
+    <t>DELTA_PROTOCOL_CHANGED (2D521)</t>
+  </si>
+  <si>
+    <t>Protocol changed by a concurrent update</t>
+  </si>
+  <si>
+    <t>A feature enabled during writes. Fix: Retry.</t>
+  </si>
+  <si>
+    <t>20, 97</t>
+  </si>
+  <si>
+    <t>UNKNOWN_FIELD_EXCEPTION (KD003)</t>
+  </si>
+  <si>
+    <t>New fields found while parsing</t>
+  </si>
+  <si>
+    <t>Auto Loader addNewColumns met a new column. Fix: Let the job restart; it resumes with the new schema.</t>
+  </si>
+  <si>
+    <t>64, 98</t>
+  </si>
+  <si>
+    <t>CLOUD_FILE_SOURCE_FILE_NOT_FOUND (42K03)</t>
+  </si>
+  <si>
+    <t>A notified file no longer exists</t>
+  </si>
+  <si>
+    <t>File deleted before it was processed. Fix: Don't delete files before they are processed.</t>
+  </si>
+  <si>
+    <t>63, 98</t>
+  </si>
+  <si>
+    <t>DELTA_SCHEMA_CHANGED (KD007)</t>
+  </si>
+  <si>
+    <t>The source schema changed under the stream</t>
+  </si>
+  <si>
+    <t>A schema change on a streamed table. Fix: Restart; if it repeats, use a new checkpoint.</t>
+  </si>
+  <si>
+    <t>65, 98</t>
+  </si>
+  <si>
+    <t>DELTA_STREAMING_INCOMPATIBLE_SCHEMA_CHANGE (42KD4)</t>
+  </si>
+  <si>
+    <t>Rename, drop or type change on a streamed table</t>
+  </si>
+  <si>
+    <t>A read-incompatible schema change. Fix: Follow the linked doc, or use a schema tracking location.</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>DELTA_SOURCE_TABLE_IGNORE_CHANGES (0A000)</t>
+  </si>
+  <si>
+    <t>An update or delete in a table read as a stream</t>
+  </si>
+  <si>
+    <t>Streams expect append-only sources. Fix: skipChangeCommits, or a fresh checkpoint / full refresh.</t>
+  </si>
+  <si>
+    <t>68, 98</t>
+  </si>
+  <si>
+    <t>DELTA_FILE_NOT_FOUND_DETAILED (42K03)</t>
+  </si>
+  <si>
+    <t>A file referenced in the log is missing</t>
+  </si>
+  <si>
+    <t>Manual deletion, or VACUUM with too short a retention. Fix: Never delete table files directly; restart with a new checkpoint.</t>
+  </si>
+  <si>
+    <t>25, 99</t>
+  </si>
+  <si>
+    <t>DELTA_VACUUM_RETENTION_PERIOD_TOO_SHORT (22003)</t>
+  </si>
+  <si>
+    <t>Retention below the safety threshold</t>
+  </si>
+  <si>
+    <t>VACUUM with a short retention. Fix: Keep at least 7 days.</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>DELTA_CANNOT_VACUUM_LITE (55000)</t>
+  </si>
+  <si>
+    <t>LITE can't find all files from the log</t>
+  </si>
+  <si>
+    <t>Untracked files in the directory. Fix: Run VACUUM FULL.</t>
+  </si>
+  <si>
+    <t>DELTA_TIMESTAMP_EARLIER_THAN_COMMIT_RETENTION (42816)</t>
+  </si>
+  <si>
+    <t>Timestamp older than the earliest kept version</t>
+  </si>
+  <si>
+    <t>History past log retention. Fix: Use a later timestamp; raise retention in advance.</t>
+  </si>
+  <si>
+    <t>24, 99</t>
+  </si>
+  <si>
+    <t>DELTA_CANNOT_RESTORE_TABLE_VERSION (22003)</t>
+  </si>
+  <si>
+    <t>Version outside the available range</t>
+  </si>
+  <si>
+    <t>Version expired or never existed. Fix: Choose a version in range.</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>DELTA_UNSUPPORTED_FEATURES_FOR_READ (56038)</t>
+  </si>
+  <si>
+    <t>Table needs reader features this runtime lacks</t>
+  </si>
+  <si>
+    <t>Feature enabled by a newer writer. Fix: Use a newer runtime or client.</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>FAILED_READ_FILE (KD001)</t>
+  </si>
+  <si>
+    <t>Error reading a file</t>
+  </si>
+  <si>
+    <t>A corrupt or unexpected file. Fix: Read the condition's details.</t>
+  </si>
+  <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>Event: compute plane network is misconfigured</t>
+  </si>
+  <si>
+    <t>Node daemon ping timeout; cluster terminated</t>
+  </si>
+  <si>
+    <t>Routing or firewall blocks the control plane. Fix: Test the path from a VM in the workspace subnet.</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>Event: METASTORE_DOWN</t>
+  </si>
+  <si>
+    <t>The metastore is unreachable from compute</t>
+  </si>
+  <si>
+    <t>A web application firewall or proxy in the path. Fix: Take the proxy out of the path.</t>
+  </si>
+  <si>
+    <t>HTTP 403 Forbidden (serverless to storage)</t>
+  </si>
+  <si>
+    <t>Serverless can't read a firewalled storage account</t>
+  </si>
+  <si>
+    <t>Allow-listed serverless subnet IDs no longer work. Fix: Network security perimeter plus the AzureDatabricksServerless tag.</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>HTTP 429 Too Many Requests (jobs)</t>
+  </si>
+  <si>
+    <t>Too many concurrent task runs</t>
+  </si>
+  <si>
+    <t>Over 2,000 concurrent task runs in a workspace. Fix: Spread or reduce concurrent runs.</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>Out of memory after a stream restart</t>
+  </si>
+  <si>
+    <t>The replanned micro-batch fails again</t>
+  </si>
+  <si>
+    <t>The batch planned before the failure is too large. Fix: Scale up the compute to get past it.</t>
+  </si>
+  <si>
+    <t>91, 98</t>
   </si>
 </sst>
 </file>
@@ -1715,7 +2337,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -4092,39 +4714,481 @@
         <v>338</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
-        <v>322</v>
+        <v>342</v>
       </c>
       <c r="B92" s="2">
         <v>91</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F92" s="2">
-        <v>10</v>
-      </c>
-      <c r="G92" s="2" t="s">
-        <v>345</v>
+        <v>3</v>
+      </c>
+      <c r="G92" s="2">
+        <v>24</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C93" s="4" t="s">
+    <row r="93" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A93" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B93" s="3">
+        <v>92</v>
+      </c>
+      <c r="C93" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="F93" s="4">
-        <f>SUM(F2:F92)</f>
-        <v>217</v>
+      <c r="D93" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F93" s="3">
+        <v>2</v>
+      </c>
+      <c r="G93" s="3">
+        <v>24</v>
+      </c>
+      <c r="H93" s="3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A94" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B94" s="2">
+        <v>93</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F94" s="2">
+        <v>2</v>
+      </c>
+      <c r="G94" s="2">
+        <v>24</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A95" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B95" s="3">
+        <v>94</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F95" s="3">
+        <v>3</v>
+      </c>
+      <c r="G95" s="3">
+        <v>24</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A96" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B96" s="2">
+        <v>95</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F96" s="2">
+        <v>2</v>
+      </c>
+      <c r="G96" s="2">
+        <v>24</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A97" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B97" s="3">
+        <v>96</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="F97" s="3">
+        <v>2</v>
+      </c>
+      <c r="G97" s="3">
+        <v>24</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A98" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B98" s="2">
+        <v>97</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F98" s="2">
+        <v>2</v>
+      </c>
+      <c r="G98" s="2">
+        <v>24</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A99" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B99" s="3">
+        <v>98</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="F99" s="3">
+        <v>3</v>
+      </c>
+      <c r="G99" s="3">
+        <v>24</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A100" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B100" s="2">
+        <v>99</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F100" s="2">
+        <v>2</v>
+      </c>
+      <c r="G100" s="2">
+        <v>24</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A101" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B101" s="3">
+        <v>100</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="F101" s="3">
+        <v>2</v>
+      </c>
+      <c r="G101" s="3">
+        <v>24</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A102" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B102" s="2">
+        <v>101</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="F102" s="2">
+        <v>2</v>
+      </c>
+      <c r="G102" s="2">
+        <v>24</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A103" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B103" s="3">
+        <v>102</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="F103" s="3">
+        <v>2</v>
+      </c>
+      <c r="G103" s="3">
+        <v>24</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A104" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B104" s="2">
+        <v>103</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="F104" s="2">
+        <v>1</v>
+      </c>
+      <c r="G104" s="2">
+        <v>24</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A105" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B105" s="3">
+        <v>104</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="F105" s="3">
+        <v>2</v>
+      </c>
+      <c r="G105" s="3">
+        <v>24</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A106" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B106" s="2">
+        <v>105</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F106" s="2">
+        <v>2</v>
+      </c>
+      <c r="G106" s="2">
+        <v>24</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+      <c r="A107" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B107" s="3">
+        <v>106</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="F107" s="3">
+        <v>3</v>
+      </c>
+      <c r="G107" s="3">
+        <v>24</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A108" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B108" s="2">
+        <v>107</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F108" s="2">
+        <v>2</v>
+      </c>
+      <c r="G108" s="2">
+        <v>24</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A109" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B109" s="3">
+        <v>108</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="F109" s="3">
+        <v>10</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C110" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F110" s="4">
+        <f>SUM(F2:F109)</f>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4134,7 +5198,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4148,45 +5212,45 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>348</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>349</v>
+        <v>418</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>350</v>
+        <v>419</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>351</v>
+        <v>420</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>353</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <f>COUNTA(B6:B96)</f>
-        <v>91</v>
+        <f>COUNTA(B6:B113)</f>
+        <v>108</v>
       </c>
       <c r="B3" s="5">
-        <f>COUNTIF(D6:D96,"Completed")</f>
+        <f>COUNTIF(D6:D113,"Completed")</f>
         <v>0</v>
       </c>
       <c r="C3" s="5">
-        <f>COUNTIF(D6:D96,"In Progress")</f>
+        <f>COUNTIF(D6:D113,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="D3" s="5">
-        <f>COUNTIF(D6:D96,"Not Started")</f>
-        <v>91</v>
+        <f>COUNTIF(D6:D113,"Not Started")</f>
+        <v>108</v>
       </c>
       <c r="E3" s="6">
-        <f>AVERAGE(E6:E96)/100</f>
+        <f>AVERAGE(E6:E113)/100</f>
         <v>0</v>
       </c>
     </row>
@@ -4201,19 +5265,19 @@
         <v>0</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>354</v>
+        <v>423</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>355</v>
+        <v>424</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>356</v>
+        <v>425</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>357</v>
+        <v>426</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>358</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -4229,7 +5293,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E6" s="2">
         <v>0</v>
@@ -4251,7 +5315,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E7" s="3">
         <v>0</v>
@@ -4273,7 +5337,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E8" s="2">
         <v>0</v>
@@ -4295,7 +5359,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E9" s="3">
         <v>0</v>
@@ -4317,7 +5381,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E10" s="2">
         <v>0</v>
@@ -4339,7 +5403,7 @@
         <v>1. Lakehouse &amp; Platform Foundations</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E11" s="3">
         <v>0</v>
@@ -4361,7 +5425,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
@@ -4383,7 +5447,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E13" s="3">
         <v>0</v>
@@ -4405,7 +5469,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E14" s="2">
         <v>0</v>
@@ -4427,7 +5491,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E15" s="3">
         <v>0</v>
@@ -4449,7 +5513,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E16" s="2">
         <v>0</v>
@@ -4471,7 +5535,7 @@
         <v>2. Parquet: The File Format</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -4493,7 +5557,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E18" s="2">
         <v>0</v>
@@ -4515,7 +5579,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E19" s="3">
         <v>0</v>
@@ -4537,7 +5601,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E20" s="2">
         <v>0</v>
@@ -4559,7 +5623,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E21" s="3">
         <v>0</v>
@@ -4581,7 +5645,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E22" s="2">
         <v>0</v>
@@ -4603,7 +5667,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E23" s="3">
         <v>0</v>
@@ -4625,7 +5689,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E24" s="2">
         <v>0</v>
@@ -4647,7 +5711,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E25" s="3">
         <v>0</v>
@@ -4669,7 +5733,7 @@
         <v>3. Delta Lake Internals</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
@@ -4691,7 +5755,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E27" s="3">
         <v>0</v>
@@ -4713,7 +5777,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E28" s="2">
         <v>0</v>
@@ -4735,7 +5799,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E29" s="3">
         <v>0</v>
@@ -4757,7 +5821,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E30" s="2">
         <v>0</v>
@@ -4779,7 +5843,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E31" s="3">
         <v>0</v>
@@ -4801,7 +5865,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -4823,7 +5887,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E33" s="3">
         <v>0</v>
@@ -4845,7 +5909,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E34" s="2">
         <v>0</v>
@@ -4867,7 +5931,7 @@
         <v>4. Delta Lake Operations</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E35" s="3">
         <v>0</v>
@@ -4889,7 +5953,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E36" s="2">
         <v>0</v>
@@ -4911,7 +5975,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E37" s="3">
         <v>0</v>
@@ -4933,7 +5997,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E38" s="2">
         <v>0</v>
@@ -4955,7 +6019,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E39" s="3">
         <v>0</v>
@@ -4977,7 +6041,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E40" s="2">
         <v>0</v>
@@ -4999,7 +6063,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E41" s="3">
         <v>0</v>
@@ -5021,7 +6085,7 @@
         <v>5. Data Layout &amp; Table Optimization</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
@@ -5043,7 +6107,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E43" s="3">
         <v>0</v>
@@ -5065,7 +6129,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E44" s="2">
         <v>0</v>
@@ -5087,7 +6151,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E45" s="3">
         <v>0</v>
@@ -5109,7 +6173,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E46" s="2">
         <v>0</v>
@@ -5131,7 +6195,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E47" s="3">
         <v>0</v>
@@ -5153,7 +6217,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E48" s="2">
         <v>0</v>
@@ -5175,7 +6239,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E49" s="3">
         <v>0</v>
@@ -5197,7 +6261,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E50" s="2">
         <v>0</v>
@@ -5219,7 +6283,7 @@
         <v>6. Unity Catalog &amp; Governance</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E51" s="3">
         <v>0</v>
@@ -5241,7 +6305,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E52" s="2">
         <v>0</v>
@@ -5263,7 +6327,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E53" s="3">
         <v>0</v>
@@ -5285,7 +6349,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E54" s="2">
         <v>0</v>
@@ -5307,7 +6371,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E55" s="3">
         <v>0</v>
@@ -5329,7 +6393,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E56" s="2">
         <v>0</v>
@@ -5351,7 +6415,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E57" s="3">
         <v>0</v>
@@ -5373,7 +6437,7 @@
         <v>7. Compute &amp; Cost</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E58" s="2">
         <v>0</v>
@@ -5395,7 +6459,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E59" s="3">
         <v>0</v>
@@ -5417,7 +6481,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E60" s="2">
         <v>0</v>
@@ -5439,7 +6503,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E61" s="3">
         <v>0</v>
@@ -5461,7 +6525,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E62" s="2">
         <v>0</v>
@@ -5483,7 +6547,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E63" s="3">
         <v>0</v>
@@ -5505,7 +6569,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E64" s="2">
         <v>0</v>
@@ -5527,7 +6591,7 @@
         <v>8. Spark &amp; Transformation</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E65" s="3">
         <v>0</v>
@@ -5549,7 +6613,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E66" s="2">
         <v>0</v>
@@ -5571,7 +6635,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E67" s="3">
         <v>0</v>
@@ -5593,7 +6657,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E68" s="2">
         <v>0</v>
@@ -5615,7 +6679,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E69" s="3">
         <v>0</v>
@@ -5637,7 +6701,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E70" s="2">
         <v>0</v>
@@ -5659,7 +6723,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E71" s="3">
         <v>0</v>
@@ -5681,7 +6745,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E72" s="2">
         <v>0</v>
@@ -5703,7 +6767,7 @@
         <v>9. Ingestion &amp; Streaming</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E73" s="3">
         <v>0</v>
@@ -5725,7 +6789,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E74" s="2">
         <v>0</v>
@@ -5747,7 +6811,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E75" s="3">
         <v>0</v>
@@ -5769,7 +6833,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E76" s="2">
         <v>0</v>
@@ -5791,7 +6855,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E77" s="3">
         <v>0</v>
@@ -5813,7 +6877,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E78" s="2">
         <v>0</v>
@@ -5835,7 +6899,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E79" s="3">
         <v>0</v>
@@ -5857,7 +6921,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E80" s="2">
         <v>0</v>
@@ -5879,7 +6943,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E81" s="3">
         <v>0</v>
@@ -5901,7 +6965,7 @@
         <v>10. Pipelines &amp; Orchestration</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E82" s="2">
         <v>0</v>
@@ -5923,7 +6987,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E83" s="3">
         <v>0</v>
@@ -5945,7 +7009,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E84" s="2">
         <v>0</v>
@@ -5967,7 +7031,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E85" s="3">
         <v>0</v>
@@ -5989,7 +7053,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E86" s="2">
         <v>0</v>
@@ -6011,7 +7075,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E87" s="3">
         <v>0</v>
@@ -6033,7 +7097,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E88" s="2">
         <v>0</v>
@@ -6055,7 +7119,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E89" s="3">
         <v>0</v>
@@ -6077,7 +7141,7 @@
         <v>11. Azure Networking for Databricks</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E90" s="2">
         <v>0</v>
@@ -6096,10 +7160,10 @@
       </c>
       <c r="C91" s="3" t="str">
         <f>'Databricks Master Syllabus'!A87</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>12. Operate &amp; Deploy</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E91" s="3">
         <v>0</v>
@@ -6118,10 +7182,10 @@
       </c>
       <c r="C92" s="2" t="str">
         <f>'Databricks Master Syllabus'!A88</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>12. Operate &amp; Deploy</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E92" s="2">
         <v>0</v>
@@ -6140,10 +7204,10 @@
       </c>
       <c r="C93" s="3" t="str">
         <f>'Databricks Master Syllabus'!A89</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>12. Operate &amp; Deploy</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E93" s="3">
         <v>0</v>
@@ -6162,10 +7226,10 @@
       </c>
       <c r="C94" s="2" t="str">
         <f>'Databricks Master Syllabus'!A90</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>12. Operate &amp; Deploy</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E94" s="2">
         <v>0</v>
@@ -6184,10 +7248,10 @@
       </c>
       <c r="C95" s="3" t="str">
         <f>'Databricks Master Syllabus'!A91</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>12. Operate &amp; Deploy</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E95" s="3">
         <v>0</v>
@@ -6202,14 +7266,14 @@
       </c>
       <c r="B96" s="2" t="str">
         <f>'Databricks Master Syllabus'!C92</f>
-        <v>Capstone: End-to-End Medallion Pipeline</v>
+        <v>Running Streams in Production</v>
       </c>
       <c r="C96" s="2" t="str">
         <f>'Databricks Master Syllabus'!A92</f>
-        <v>12. Operate, Deploy &amp; Capstone</v>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="E96" s="2">
         <v>0</v>
@@ -6217,6 +7281,380 @@
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
+    </row>
+    <row r="97" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A97" s="3">
+        <v>92</v>
+      </c>
+      <c r="B97" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C93</f>
+        <v>Stateful Streaming in Production</v>
+      </c>
+      <c r="C97" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A93</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E97" s="3">
+        <v>0</v>
+      </c>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+    </row>
+    <row r="98" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A98" s="2">
+        <v>93</v>
+      </c>
+      <c r="B98" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C94</f>
+        <v>Notifications and Alerts</v>
+      </c>
+      <c r="C98" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A94</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E98" s="2">
+        <v>0</v>
+      </c>
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
+      <c r="H98" s="2"/>
+    </row>
+    <row r="99" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A99" s="3">
+        <v>94</v>
+      </c>
+      <c r="B99" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C95</f>
+        <v>Troubleshooting a Failed Job</v>
+      </c>
+      <c r="C99" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A95</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E99" s="3">
+        <v>0</v>
+      </c>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+    </row>
+    <row r="100" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
+        <v>95</v>
+      </c>
+      <c r="B100" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C96</f>
+        <v>Reading Errors: Conditions and SQLSTATE</v>
+      </c>
+      <c r="C100" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A96</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E100" s="2">
+        <v>0</v>
+      </c>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
+      <c r="H100" s="2"/>
+    </row>
+    <row r="101" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A101" s="3">
+        <v>96</v>
+      </c>
+      <c r="B101" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C97</f>
+        <v>Write, Schema and MERGE Errors</v>
+      </c>
+      <c r="C101" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A97</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E101" s="3">
+        <v>0</v>
+      </c>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+    </row>
+    <row r="102" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A102" s="2">
+        <v>97</v>
+      </c>
+      <c r="B102" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C98</f>
+        <v>Concurrent Write Conflicts</v>
+      </c>
+      <c r="C102" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A98</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E102" s="2">
+        <v>0</v>
+      </c>
+      <c r="F102" s="2"/>
+      <c r="G102" s="2"/>
+      <c r="H102" s="2"/>
+    </row>
+    <row r="103" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A103" s="3">
+        <v>98</v>
+      </c>
+      <c r="B103" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C99</f>
+        <v>Streaming Errors</v>
+      </c>
+      <c r="C103" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A99</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E103" s="3">
+        <v>0</v>
+      </c>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+    </row>
+    <row r="104" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A104" s="2">
+        <v>99</v>
+      </c>
+      <c r="B104" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C100</f>
+        <v>File, History and Retention Errors</v>
+      </c>
+      <c r="C104" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A100</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E104" s="2">
+        <v>0</v>
+      </c>
+      <c r="F104" s="2"/>
+      <c r="G104" s="2"/>
+      <c r="H104" s="2"/>
+    </row>
+    <row r="105" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A105" s="3">
+        <v>100</v>
+      </c>
+      <c r="B105" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C101</f>
+        <v>Query Profile and Query History</v>
+      </c>
+      <c r="C105" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A101</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E105" s="3">
+        <v>0</v>
+      </c>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+    </row>
+    <row r="106" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A106" s="2">
+        <v>101</v>
+      </c>
+      <c r="B106" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C102</f>
+        <v>Compute That Won't Start</v>
+      </c>
+      <c r="C106" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A102</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E106" s="2">
+        <v>0</v>
+      </c>
+      <c r="F106" s="2"/>
+      <c r="G106" s="2"/>
+      <c r="H106" s="2"/>
+    </row>
+    <row r="107" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A107" s="3">
+        <v>102</v>
+      </c>
+      <c r="B107" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C103</f>
+        <v>Libraries and Init Scripts</v>
+      </c>
+      <c r="C107" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A103</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E107" s="3">
+        <v>0</v>
+      </c>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+    </row>
+    <row r="108" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A108" s="2">
+        <v>103</v>
+      </c>
+      <c r="B108" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C104</f>
+        <v>Runtime Lifecycle and Upgrades</v>
+      </c>
+      <c r="C108" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A104</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E108" s="2">
+        <v>0</v>
+      </c>
+      <c r="F108" s="2"/>
+      <c r="G108" s="2"/>
+      <c r="H108" s="2"/>
+    </row>
+    <row r="109" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A109" s="3">
+        <v>104</v>
+      </c>
+      <c r="B109" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C105</f>
+        <v>Environment Isolation and Catalog Strategy</v>
+      </c>
+      <c r="C109" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A105</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E109" s="3">
+        <v>0</v>
+      </c>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+    </row>
+    <row r="110" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A110" s="2">
+        <v>105</v>
+      </c>
+      <c r="B110" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C106</f>
+        <v>Encryption and Customer-Managed Keys</v>
+      </c>
+      <c r="C110" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A106</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E110" s="2">
+        <v>0</v>
+      </c>
+      <c r="F110" s="2"/>
+      <c r="G110" s="2"/>
+      <c r="H110" s="2"/>
+    </row>
+    <row r="111" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A111" s="3">
+        <v>106</v>
+      </c>
+      <c r="B111" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C107</f>
+        <v>High Availability and Disaster Recovery</v>
+      </c>
+      <c r="C111" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A107</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E111" s="3">
+        <v>0</v>
+      </c>
+      <c r="F111" s="3"/>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+    </row>
+    <row r="112" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A112" s="2">
+        <v>107</v>
+      </c>
+      <c r="B112" s="2" t="str">
+        <f>'Databricks Master Syllabus'!C108</f>
+        <v>Testing Databricks Code</v>
+      </c>
+      <c r="C112" s="2" t="str">
+        <f>'Databricks Master Syllabus'!A108</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E112" s="2">
+        <v>0</v>
+      </c>
+      <c r="F112" s="2"/>
+      <c r="G112" s="2"/>
+      <c r="H112" s="2"/>
+    </row>
+    <row r="113" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+      <c r="A113" s="3">
+        <v>108</v>
+      </c>
+      <c r="B113" s="3" t="str">
+        <f>'Databricks Master Syllabus'!C109</f>
+        <v>Capstone: End-to-End Medallion Pipeline</v>
+      </c>
+      <c r="C113" s="3" t="str">
+        <f>'Databricks Master Syllabus'!A109</f>
+        <v>13. Production, Troubleshooting &amp; Capstone</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E113" s="3">
+        <v>0</v>
+      </c>
+      <c r="F113" s="3"/>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6235,178 +7673,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>359</v>
+        <v>428</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>360</v>
+        <v>429</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>361</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>362</v>
+        <v>431</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>363</v>
+        <v>432</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>364</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>365</v>
+        <v>434</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>366</v>
+        <v>435</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>367</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>368</v>
+        <v>437</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>369</v>
+        <v>438</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>370</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>371</v>
+        <v>440</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>372</v>
+        <v>441</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>373</v>
+        <v>442</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>374</v>
+        <v>443</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>375</v>
+        <v>444</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>376</v>
+        <v>445</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>377</v>
+        <v>446</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>378</v>
+        <v>447</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>376</v>
+        <v>445</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>379</v>
+        <v>448</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>380</v>
+        <v>449</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>376</v>
+        <v>445</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>381</v>
+        <v>450</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>382</v>
+        <v>451</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>383</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>384</v>
+        <v>453</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>385</v>
+        <v>454</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>386</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>387</v>
+        <v>456</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>388</v>
+        <v>457</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>389</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>390</v>
+        <v>459</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>391</v>
+        <v>460</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>392</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>393</v>
+        <v>462</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>394</v>
+        <v>463</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>392</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>395</v>
+        <v>464</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>396</v>
+        <v>465</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>397</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>398</v>
+        <v>467</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>399</v>
+        <v>468</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>376</v>
+        <v>445</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>400</v>
+        <v>469</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>401</v>
+        <v>470</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>402</v>
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -6425,66 +7863,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>403</v>
+        <v>472</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>404</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>405</v>
+        <v>474</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>406</v>
+        <v>475</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>407</v>
+        <v>476</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>408</v>
+        <v>477</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>409</v>
+        <v>478</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>410</v>
+        <v>479</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>411</v>
+        <v>480</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>412</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>413</v>
+        <v>482</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>414</v>
+        <v>483</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>415</v>
+        <v>484</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>416</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>417</v>
+        <v>486</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>418</v>
+        <v>487</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="28" x14ac:dyDescent="0.35">
@@ -6492,63 +7930,583 @@
         <v>102</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>419</v>
+        <v>488</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>371</v>
+        <v>440</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>420</v>
+        <v>489</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="28" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>421</v>
+        <v>490</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>422</v>
+        <v>491</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>423</v>
+        <v>492</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>424</v>
+        <v>493</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>425</v>
+        <v>494</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>426</v>
+        <v>495</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>427</v>
+        <v>496</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>428</v>
+        <v>497</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>429</v>
+        <v>498</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>430</v>
+        <v>499</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>431</v>
+        <v>500</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>432</v>
+        <v>501</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build the Databricks study guide (pack databricks v1, 24 chapters)
24 chapters written as Markdown and built into v1.json: the lakehouse,
Parquet, Delta internals, history and VACUUM, schemas, MERGE and change data
feed, data layout, Unity Catalog, tables and storage, access control,
compute, Spark, medallion, ingestion, Auto Loader, streaming, declarative
pipelines, jobs, performance, monitoring, CI/CD, ADF and ADLS, Azure
networking and production. Each opens with its alignment to the 108-topic
roadmap, cites the research notes, has Free Edition steps where Free Edition
can run them, and ends with a trade-off and an interview takeaway. Four
figures. test_databricks_pack.py holds the guide to the workbook and the
notes; the pack joins the shared content-pack tests. Axe (light and dark)
and 390px checks passed on all 25 guide pages against a scratch database.
</commit_message>
<xml_diff>
--- a/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
+++ b/docs/research/Databricks_Data_Engineering_Mastery_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\PrepBench\.claude\worktrees\databricks-research-1e243f\docs\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4230A312-1C88-4DD3-BD53-B23662758D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6328D6D0-0052-413C-AE5B-E3F1F747CDD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,7 +219,7 @@
     <t>Understand Delta Lake as Parquet data files plus a file-based transaction log, and that every Databricks table is Delta by default.</t>
   </si>
   <si>
-    <t>Create a Delta table, list its directory, and point out the data files and the _delta_log folder.</t>
+    <t>Create a Delta table and use DESCRIBE DETAIL to show its location, file count and protocol, then explain what its _delta_log folder holds.</t>
   </si>
   <si>
     <t>§2.1</t>
@@ -231,7 +231,7 @@
     <t>Master the log: one JSON file per version, 20-digit zero-padded names, contiguous versions, a version's file as the unit of atomicity.</t>
   </si>
   <si>
-    <t>Make three writes, open the three JSON commits, and name the version each one created.</t>
+    <t>Make three writes, list them with DESCRIBE HISTORY, and name the version and JSON commit file each one created.</t>
   </si>
   <si>
     <t>Log Actions</t>
@@ -2686,7 +2686,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>57</v>
       </c>

</xml_diff>